<commit_message>
Work on <design drawIO
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_debugCL42T\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_designHRTIM\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F3F433-34F5-4C18-84B3-6F13E4CA76C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15595E55-9134-45ED-9550-FDC200154CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="FMKCAN" sheetId="7" r:id="rId6"/>
     <sheet name="FMKSRL" sheetId="8" r:id="rId7"/>
     <sheet name="Feuil1" sheetId="5" r:id="rId8"/>
+    <sheet name="Feuil2" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="455">
   <si>
     <t>Colonne1</t>
   </si>
@@ -1002,9 +1003,6 @@
     <t>PWM</t>
   </si>
   <si>
-    <t>EVNT</t>
-  </si>
-  <si>
     <t>periodMs</t>
   </si>
   <si>
@@ -1366,13 +1364,58 @@
   </si>
   <si>
     <t>;</t>
+  </si>
+  <si>
+    <t>HRTIM</t>
+  </si>
+  <si>
+    <t>MUL32</t>
+  </si>
+  <si>
+    <t>MUL16</t>
+  </si>
+  <si>
+    <t>MUL8</t>
+  </si>
+  <si>
+    <t>MUL4</t>
+  </si>
+  <si>
+    <t>MUL2</t>
+  </si>
+  <si>
+    <t>DIV1</t>
+  </si>
+  <si>
+    <t>DIV2</t>
+  </si>
+  <si>
+    <t>DIV4</t>
+  </si>
+  <si>
+    <t>Prescaler Ratio</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clockSystem </t>
+  </si>
+  <si>
+    <t>Min ARR</t>
+  </si>
+  <si>
+    <t>Max ARR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1393,8 +1436,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1413,8 +1464,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1422,11 +1485,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1438,11 +1541,179 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -4086,6 +4357,32 @@
 </table>
 </file>
 
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{9E5B015E-0B8D-49DB-8A74-4F6D1452471D}" name="Tableau20" displayName="Tableau20" ref="E7:G15" totalsRowShown="0">
+  <autoFilter ref="E7:G15" xr:uid="{9E5B015E-0B8D-49DB-8A74-4F6D1452471D}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{094F0F32-9797-4DD4-934E-F3C2C577DF5D}" name="Prescaler Ratio"/>
+    <tableColumn id="2" xr3:uid="{7661070E-E3D3-4CB7-B8A8-67A52F24F99B}" name="Min" dataDxfId="8">
+      <calculatedColumnFormula>$J$6 *$O$8 / $K$6</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{AF4C7D4D-6C03-4435-85F8-25E20A9543BE}" name="Max"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{234B95CE-5663-49A6-97EA-930C7F4E968E}" name="Tableau21" displayName="Tableau21" ref="E20:G28" totalsRowShown="0" headerRowDxfId="7" dataDxfId="5" headerRowBorderDxfId="6" tableBorderDxfId="4" totalsRowBorderDxfId="3">
+  <autoFilter ref="E20:G28" xr:uid="{234B95CE-5663-49A6-97EA-930C7F4E968E}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{4F0EEA58-CD5B-4B51-B80B-81B99A5A2326}" name="Prescaler Ratio" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{A7EA45FD-C73A-4CE6-B221-0EDC312BC096}" name="Max" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{C80C0705-52C9-4BF1-97DD-0B75B2A7CCC7}" name="Min" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5A8C957F-EDE6-44F1-B8F8-2086E255196A}" name="GI_DAC" displayName="GI_DAC" ref="Y36:Z37" totalsRowShown="0">
   <autoFilter ref="Y36:Z37" xr:uid="{5A8C957F-EDE6-44F1-B8F8-2086E255196A}"/>
@@ -4507,7 +4804,7 @@
         <v>297</v>
       </c>
       <c r="F18" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="H18" t="s">
         <v>57</v>
@@ -4542,7 +4839,7 @@
         <v>304</v>
       </c>
       <c r="F19" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H19" t="s">
         <v>59</v>
@@ -4574,7 +4871,7 @@
         <v>304</v>
       </c>
       <c r="F20" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H20" t="s">
         <v>124</v>
@@ -4627,7 +4924,7 @@
         <v>304</v>
       </c>
       <c r="F21" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H21" t="s">
         <v>125</v>
@@ -4663,7 +4960,7 @@
         <v>237</v>
       </c>
       <c r="AB21" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AC21">
         <v>8</v>
@@ -4680,7 +4977,7 @@
         <v>304</v>
       </c>
       <c r="F22" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H22" t="s">
         <v>126</v>
@@ -4716,7 +5013,7 @@
         <v>237</v>
       </c>
       <c r="AB22" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="AC22">
         <v>8</v>
@@ -4733,7 +5030,7 @@
         <v>304</v>
       </c>
       <c r="F23" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H23" t="s">
         <v>60</v>
@@ -4777,7 +5074,7 @@
         <v>304</v>
       </c>
       <c r="F24" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H24" t="s">
         <v>61</v>
@@ -4821,7 +5118,7 @@
         <v>304</v>
       </c>
       <c r="F25" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H25" t="s">
         <v>127</v>
@@ -4865,7 +5162,7 @@
         <v>305</v>
       </c>
       <c r="F26" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H26" t="s">
         <v>128</v>
@@ -4903,7 +5200,7 @@
         <v>305</v>
       </c>
       <c r="F27" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H27" t="s">
         <v>129</v>
@@ -4941,7 +5238,7 @@
         <v>305</v>
       </c>
       <c r="F28" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H28" t="s">
         <v>130</v>
@@ -4979,7 +5276,7 @@
         <v>305</v>
       </c>
       <c r="F29" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H29" t="s">
         <v>131</v>
@@ -5011,7 +5308,7 @@
         <v>305</v>
       </c>
       <c r="F30" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H30" t="s">
         <v>62</v>
@@ -5043,7 +5340,7 @@
         <v>305</v>
       </c>
       <c r="F31" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H31" t="s">
         <v>132</v>
@@ -5060,7 +5357,7 @@
         <v>305</v>
       </c>
       <c r="F32" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H32" t="s">
         <v>133</v>
@@ -5077,7 +5374,7 @@
         <v>303</v>
       </c>
       <c r="F33" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H33" t="s">
         <v>134</v>
@@ -5100,7 +5397,7 @@
         <v>303</v>
       </c>
       <c r="F34" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H34" t="s">
         <v>135</v>
@@ -5123,7 +5420,7 @@
         <v>295</v>
       </c>
       <c r="F35" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H35" t="s">
         <v>136</v>
@@ -5146,7 +5443,7 @@
         <v>295</v>
       </c>
       <c r="F36" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H36" t="s">
         <v>137</v>
@@ -5175,7 +5472,7 @@
         <v>295</v>
       </c>
       <c r="F37" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H37" t="s">
         <v>138</v>
@@ -5204,7 +5501,7 @@
         <v>295</v>
       </c>
       <c r="F38" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H38" t="s">
         <v>139</v>
@@ -5227,7 +5524,7 @@
         <v>305</v>
       </c>
       <c r="F39" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H39" t="s">
         <v>140</v>
@@ -5250,7 +5547,7 @@
         <v>305</v>
       </c>
       <c r="F40" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H40" t="s">
         <v>141</v>
@@ -5276,7 +5573,7 @@
         <v>302</v>
       </c>
       <c r="F41" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H41" t="s">
         <v>142</v>
@@ -5296,7 +5593,7 @@
         <v>294</v>
       </c>
       <c r="F42" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H42" t="s">
         <v>143</v>
@@ -5316,7 +5613,7 @@
         <v>294</v>
       </c>
       <c r="F43" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H43" t="s">
         <v>144</v>
@@ -5336,7 +5633,7 @@
         <v>294</v>
       </c>
       <c r="F44" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H44" t="s">
         <v>145</v>
@@ -5353,7 +5650,7 @@
         <v>294</v>
       </c>
       <c r="F45" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H45" t="s">
         <v>146</v>
@@ -5370,7 +5667,7 @@
         <v>294</v>
       </c>
       <c r="F46" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H46" t="s">
         <v>63</v>
@@ -5390,7 +5687,7 @@
         <v>294</v>
       </c>
       <c r="F47" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H47" t="s">
         <v>147</v>
@@ -5410,7 +5707,7 @@
         <v>294</v>
       </c>
       <c r="F48" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H48" t="s">
         <v>64</v>
@@ -5430,7 +5727,7 @@
         <v>294</v>
       </c>
       <c r="F49" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H49" t="s">
         <v>148</v>
@@ -5450,7 +5747,7 @@
         <v>294</v>
       </c>
       <c r="F50" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H50" t="s">
         <v>149</v>
@@ -5467,7 +5764,7 @@
         <v>294</v>
       </c>
       <c r="F51" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H51" t="s">
         <v>150</v>
@@ -5484,7 +5781,7 @@
         <v>294</v>
       </c>
       <c r="F52" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H52" t="s">
         <v>151</v>
@@ -5504,7 +5801,7 @@
         <v>294</v>
       </c>
       <c r="F53" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H53" t="s">
         <v>152</v>
@@ -5524,7 +5821,7 @@
         <v>294</v>
       </c>
       <c r="F54" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H54" t="s">
         <v>65</v>
@@ -5544,7 +5841,7 @@
         <v>294</v>
       </c>
       <c r="F55" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H55" t="s">
         <v>66</v>
@@ -5564,7 +5861,7 @@
         <v>294</v>
       </c>
       <c r="F56" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H56" t="s">
         <v>67</v>
@@ -5584,7 +5881,7 @@
         <v>294</v>
       </c>
       <c r="F57" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H57" t="s">
         <v>68</v>
@@ -5604,7 +5901,7 @@
         <v>294</v>
       </c>
       <c r="F58" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H58" t="s">
         <v>153</v>
@@ -5624,7 +5921,7 @@
         <v>302</v>
       </c>
       <c r="F59" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H59" t="s">
         <v>154</v>
@@ -5644,7 +5941,7 @@
         <v>294</v>
       </c>
       <c r="F60" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H60" t="s">
         <v>155</v>
@@ -5664,7 +5961,7 @@
         <v>294</v>
       </c>
       <c r="F61" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H61" t="s">
         <v>156</v>
@@ -5684,7 +5981,7 @@
         <v>294</v>
       </c>
       <c r="F62" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H62" t="s">
         <v>157</v>
@@ -5704,7 +6001,7 @@
         <v>294</v>
       </c>
       <c r="F63" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H63" t="s">
         <v>158</v>
@@ -5721,7 +6018,7 @@
         <v>295</v>
       </c>
       <c r="F64" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H64" t="s">
         <v>159</v>
@@ -5738,7 +6035,7 @@
         <v>295</v>
       </c>
       <c r="F65" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H65" t="s">
         <v>160</v>
@@ -5755,7 +6052,7 @@
         <v>295</v>
       </c>
       <c r="F66" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H66" t="s">
         <v>161</v>
@@ -5772,7 +6069,7 @@
         <v>295</v>
       </c>
       <c r="F67" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H67" t="s">
         <v>162</v>
@@ -5789,7 +6086,7 @@
         <v>295</v>
       </c>
       <c r="F68" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H68" t="s">
         <v>163</v>
@@ -5806,7 +6103,7 @@
         <v>295</v>
       </c>
       <c r="F69" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H69" t="s">
         <v>164</v>
@@ -5823,7 +6120,7 @@
         <v>295</v>
       </c>
       <c r="F70" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H70" t="s">
         <v>165</v>
@@ -5840,7 +6137,7 @@
         <v>295</v>
       </c>
       <c r="F71" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H71" t="s">
         <v>166</v>
@@ -5857,7 +6154,7 @@
         <v>295</v>
       </c>
       <c r="F72" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H72" t="s">
         <v>167</v>
@@ -5874,7 +6171,7 @@
         <v>295</v>
       </c>
       <c r="F73" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H73" t="s">
         <v>168</v>
@@ -5891,7 +6188,7 @@
         <v>295</v>
       </c>
       <c r="F74" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H74" t="s">
         <v>169</v>
@@ -5908,7 +6205,7 @@
         <v>295</v>
       </c>
       <c r="F75" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H75" t="s">
         <v>170</v>
@@ -6339,10 +6636,10 @@
   <sheetData>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
@@ -6471,7 +6768,7 @@
         <v>34</v>
       </c>
       <c r="R7" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="S7" t="s">
         <v>4</v>
@@ -6486,7 +6783,7 @@
         <v>27</v>
       </c>
       <c r="X7" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="Z7" t="s">
         <v>23</v>
@@ -6536,7 +6833,7 @@
         <v>35</v>
       </c>
       <c r="R8" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="S8" t="s">
         <v>4</v>
@@ -6551,7 +6848,7 @@
         <v>30</v>
       </c>
       <c r="X8" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="Z8" t="s">
         <v>12</v>
@@ -6601,7 +6898,7 @@
         <v>27</v>
       </c>
       <c r="R9" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="S9" t="s">
         <v>256</v>
@@ -6657,7 +6954,7 @@
         <v>28</v>
       </c>
       <c r="R10" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="S10" t="s">
         <v>4</v>
@@ -6698,7 +6995,7 @@
         <v>31</v>
       </c>
       <c r="R11" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="S11" t="s">
         <v>255</v>
@@ -6727,7 +7024,7 @@
         <v>32</v>
       </c>
       <c r="R12" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="S12" t="s">
         <v>255</v>
@@ -6756,7 +7053,7 @@
         <v>33</v>
       </c>
       <c r="R13" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="S13" t="s">
         <v>256</v>
@@ -6785,7 +7082,7 @@
         <v>34</v>
       </c>
       <c r="R14" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="S14" t="s">
         <v>255</v>
@@ -6808,7 +7105,7 @@
         <v>31</v>
       </c>
       <c r="R15" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="S15" t="s">
         <v>252</v>
@@ -6831,7 +7128,7 @@
         <v>32</v>
       </c>
       <c r="R16" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="S16" t="s">
         <v>252</v>
@@ -6854,7 +7151,7 @@
         <v>33</v>
       </c>
       <c r="R17" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="S17" t="s">
         <v>252</v>
@@ -6871,7 +7168,7 @@
         <v>34</v>
       </c>
       <c r="R18" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="S18" t="s">
         <v>252</v>
@@ -6882,7 +7179,7 @@
     </row>
     <row r="24" spans="1:53" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="25" spans="1:53" x14ac:dyDescent="0.3">
@@ -6965,12 +7262,12 @@
         <v>290</v>
       </c>
       <c r="W28" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="29" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W29" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="AW29" t="s">
         <v>91</v>
@@ -6981,7 +7278,7 @@
     </row>
     <row r="30" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W30" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AW30" t="s">
         <v>25</v>
@@ -6995,7 +7292,7 @@
     </row>
     <row r="31" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W31" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AW31" t="s">
         <v>26</v>
@@ -7009,7 +7306,7 @@
     </row>
     <row r="32" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W32" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AW32" t="s">
         <v>27</v>
@@ -7023,10 +7320,10 @@
     </row>
     <row r="33" spans="1:53" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="W33" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AW33" t="s">
         <v>28</v>
@@ -7055,10 +7352,10 @@
         <v>42</v>
       </c>
       <c r="F34" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="W34" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AW34" t="s">
         <v>29</v>
@@ -7084,13 +7381,13 @@
         <v>27</v>
       </c>
       <c r="E35" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F35" t="s">
         <v>79</v>
       </c>
       <c r="W35" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AW35" t="s">
         <v>30</v>
@@ -7113,13 +7410,13 @@
         <v>35</v>
       </c>
       <c r="E36" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="F36" t="s">
         <v>277</v>
       </c>
       <c r="W36" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="AW36" t="s">
         <v>31</v>
@@ -7287,7 +7584,7 @@
         <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
@@ -7298,10 +7595,10 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="G4" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
@@ -7312,7 +7609,7 @@
         <v>45</v>
       </c>
       <c r="F5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="G5" t="s">
         <v>6</v>
@@ -7326,7 +7623,7 @@
         <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G6" t="s">
         <v>7</v>
@@ -7334,7 +7631,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="G7" t="s">
         <v>8</v>
@@ -7342,7 +7639,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G8" t="s">
         <v>4</v>
@@ -7350,7 +7647,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G9" t="s">
         <v>251</v>
@@ -7358,7 +7655,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G10" t="s">
         <v>5</v>
@@ -7366,7 +7663,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G11" t="s">
         <v>252</v>
@@ -7374,7 +7671,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="G12" t="s">
         <v>253</v>
@@ -7382,7 +7679,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G13" t="s">
         <v>254</v>
@@ -7390,7 +7687,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="G14" t="s">
         <v>255</v>
@@ -7398,7 +7695,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F15" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="G15" t="s">
         <v>256</v>
@@ -7406,7 +7703,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F16" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G16" t="s">
         <v>256</v>
@@ -7414,7 +7711,7 @@
     </row>
     <row r="17" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F17" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="G17" t="s">
         <v>256</v>
@@ -7496,7 +7793,7 @@
         <v>110</v>
       </c>
       <c r="S4" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="T4" t="s">
         <v>268</v>
@@ -7522,7 +7819,7 @@
         <v>98</v>
       </c>
       <c r="S5" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="T5" t="s">
         <v>268</v>
@@ -7536,7 +7833,7 @@
     </row>
     <row r="6" spans="5:22" x14ac:dyDescent="0.3">
       <c r="S6" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="T6" t="s">
         <v>268</v>
@@ -7550,10 +7847,10 @@
     </row>
     <row r="7" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="S7" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="T7" t="s">
         <v>268</v>
@@ -7567,13 +7864,13 @@
     </row>
     <row r="8" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="F8" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="S8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="T8" t="s">
         <v>268</v>
@@ -7587,34 +7884,34 @@
     </row>
     <row r="9" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F9" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="10" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="F10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="11" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F11" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="12" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F12" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -7661,50 +7958,50 @@
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
+        <v>333</v>
+      </c>
+      <c r="C2" t="s">
         <v>334</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>335</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>336</v>
       </c>
-      <c r="E2" t="s">
-        <v>337</v>
-      </c>
       <c r="J2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
+        <v>330</v>
+      </c>
+      <c r="C3" t="s">
         <v>331</v>
       </c>
-      <c r="C3" t="s">
-        <v>332</v>
-      </c>
       <c r="D3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E3" t="s">
         <v>69</v>
       </c>
       <c r="J3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="K3" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="P3" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C4" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D4" t="s">
         <v>50</v>
@@ -7713,13 +8010,13 @@
         <v>69</v>
       </c>
       <c r="J4" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="L4" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="P4" t="s">
         <v>233</v>
@@ -7727,10 +8024,10 @@
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D5" t="s">
         <v>92</v>
@@ -7739,18 +8036,18 @@
         <v>69</v>
       </c>
       <c r="J5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="K5" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C6" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D6" t="s">
         <v>45</v>
@@ -7759,18 +8056,18 @@
         <v>69</v>
       </c>
       <c r="J6" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="K6" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D7" t="s">
         <v>46</v>
@@ -7779,58 +8076,58 @@
         <v>69</v>
       </c>
       <c r="J7" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="K7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C8" t="s">
+        <v>331</v>
+      </c>
+      <c r="D8" t="s">
         <v>341</v>
-      </c>
-      <c r="C8" t="s">
-        <v>332</v>
-      </c>
-      <c r="D8" t="s">
-        <v>342</v>
       </c>
       <c r="E8" t="s">
         <v>69</v>
       </c>
       <c r="J8" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="K8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
+        <v>342</v>
+      </c>
+      <c r="C9" t="s">
+        <v>331</v>
+      </c>
+      <c r="D9" t="s">
         <v>343</v>
-      </c>
-      <c r="C9" t="s">
-        <v>332</v>
-      </c>
-      <c r="D9" t="s">
-        <v>344</v>
       </c>
       <c r="E9" t="s">
         <v>69</v>
       </c>
       <c r="J9" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="K9" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D10" t="s">
         <v>46</v>
@@ -7839,18 +8136,18 @@
         <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="K10" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C11" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D11" t="s">
         <v>45</v>
@@ -7859,18 +8156,18 @@
         <v>69</v>
       </c>
       <c r="J11" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="K11" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D12" t="s">
         <v>92</v>
@@ -7879,43 +8176,43 @@
         <v>69</v>
       </c>
       <c r="J12" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="K12" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J13" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="K13" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J14" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J15" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J16" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J17" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="18" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J18" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -7935,47 +8232,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -8005,16 +8302,16 @@
   <sheetData>
     <row r="2" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G2" t="s">
+        <v>418</v>
+      </c>
+      <c r="H2" t="s">
         <v>419</v>
-      </c>
-      <c r="H2" t="s">
-        <v>420</v>
       </c>
       <c r="I2" t="s">
         <v>285</v>
@@ -8037,7 +8334,7 @@
         <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -8058,7 +8355,7 @@
         <v>29</v>
       </c>
       <c r="M3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="4" spans="5:13" x14ac:dyDescent="0.3">
@@ -8066,7 +8363,7 @@
         <v>79</v>
       </c>
       <c r="F4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G4">
         <v>256</v>
@@ -8087,7 +8384,7 @@
         <v>27</v>
       </c>
       <c r="M4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="5:13" x14ac:dyDescent="0.3">
@@ -8095,7 +8392,7 @@
         <v>219</v>
       </c>
       <c r="F5" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="I5" t="s">
         <v>259</v>
@@ -8110,7 +8407,7 @@
         <v>31</v>
       </c>
       <c r="M5" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="6" spans="5:13" x14ac:dyDescent="0.3">
@@ -8118,7 +8415,7 @@
         <v>277</v>
       </c>
       <c r="F6" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="G6">
         <v>256</v>
@@ -8139,7 +8436,7 @@
         <v>33</v>
       </c>
       <c r="M6" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="7" spans="5:13" x14ac:dyDescent="0.3">
@@ -8147,7 +8444,7 @@
         <v>278</v>
       </c>
       <c r="F7" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -8168,7 +8465,7 @@
         <v>35</v>
       </c>
       <c r="M7" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
   </sheetData>
@@ -8341,17 +8638,12 @@
       <c r="N23" s="5"/>
       <c r="O23" s="5"/>
     </row>
-    <row r="27" spans="2:16" ht="93.6" x14ac:dyDescent="1.75">
-      <c r="D27" s="6" t="s">
-        <v>319</v>
-      </c>
-    </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D28" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="K28" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.3">
@@ -8368,34 +8660,34 @@
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D30" t="s">
+        <v>319</v>
+      </c>
+      <c r="E30" t="s">
         <v>320</v>
       </c>
-      <c r="E30" t="s">
-        <v>321</v>
-      </c>
       <c r="F30" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G30" t="s">
         <v>307</v>
       </c>
       <c r="I30" t="s">
+        <v>326</v>
+      </c>
+      <c r="J30" t="s">
+        <v>324</v>
+      </c>
+      <c r="K30" t="s">
         <v>327</v>
       </c>
-      <c r="J30" t="s">
+      <c r="L30" t="s">
+        <v>328</v>
+      </c>
+      <c r="M30" t="s">
         <v>325</v>
       </c>
-      <c r="K30" t="s">
-        <v>328</v>
-      </c>
-      <c r="L30" t="s">
+      <c r="O30" t="s">
         <v>329</v>
-      </c>
-      <c r="M30" t="s">
-        <v>326</v>
-      </c>
-      <c r="O30" t="s">
-        <v>330</v>
       </c>
       <c r="P30" t="e">
         <f>2^#REF!</f>
@@ -15122,4 +15414,271 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34ECC9F7-B649-41BF-A742-3CCEA0266A56}">
+  <dimension ref="B3:O28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="18.77734375" customWidth="1"/>
+    <col min="6" max="6" width="20.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:15" ht="93.6" x14ac:dyDescent="1.75">
+      <c r="B3" s="6" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="J5" t="s">
+        <v>452</v>
+      </c>
+      <c r="K5" t="s">
+        <v>453</v>
+      </c>
+      <c r="L5" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="J6">
+        <v>128000000</v>
+      </c>
+      <c r="K6">
+        <v>1024</v>
+      </c>
+      <c r="L6">
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>449</v>
+      </c>
+      <c r="F7" t="s">
+        <v>450</v>
+      </c>
+      <c r="G7" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
+        <v>441</v>
+      </c>
+      <c r="F8">
+        <f t="shared" ref="F8:F15" si="0">$J$6 *$O$8 / $K$6</f>
+        <v>4000000</v>
+      </c>
+      <c r="O8">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>442</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>4000000</v>
+      </c>
+      <c r="O9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>443</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>4000000</v>
+      </c>
+      <c r="O10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>444</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>4000000</v>
+      </c>
+      <c r="O11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>445</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>4000000</v>
+      </c>
+      <c r="O12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>446</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>4000000</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="E14" t="s">
+        <v>447</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>4000000</v>
+      </c>
+      <c r="O14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="E15" t="s">
+        <v>448</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>4000000</v>
+      </c>
+      <c r="O15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E20" s="9" t="s">
+        <v>449</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="21" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E21" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="F21" s="7">
+        <f>$J$6 *$O$8 / $K$6</f>
+        <v>4000000</v>
+      </c>
+      <c r="G21" s="7">
+        <f>$J$6 *$O$8 / $L$6</f>
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="22" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E22" s="8" t="s">
+        <v>442</v>
+      </c>
+      <c r="F22" s="8">
+        <f>$J$6 *$O$9 / $K$6</f>
+        <v>2000000</v>
+      </c>
+      <c r="G22" s="8">
+        <f>$J$6 *$O$9 / $L$6</f>
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="23" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E23" s="7" t="s">
+        <v>443</v>
+      </c>
+      <c r="F23" s="7">
+        <f>$J$6 *$O$10 / $K$6</f>
+        <v>1000000</v>
+      </c>
+      <c r="G23" s="7">
+        <f>$J$6 *$O$10 / $L$6</f>
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="24" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E24" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="F24" s="8">
+        <f>$J$6 *$O$11 / $K$6</f>
+        <v>500000</v>
+      </c>
+      <c r="G24" s="8">
+        <f>$J$6 *$O$11 / $L$6</f>
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="25" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E25" s="7" t="s">
+        <v>445</v>
+      </c>
+      <c r="F25" s="7">
+        <f>$J$6 *$O$12 / $K$6</f>
+        <v>250000</v>
+      </c>
+      <c r="G25" s="7">
+        <f>$J$6 *$O$12 / $L$6</f>
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="26" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E26" s="8" t="s">
+        <v>446</v>
+      </c>
+      <c r="F26" s="8">
+        <f>$J$6 *$O$13 / $K$6</f>
+        <v>125000</v>
+      </c>
+      <c r="G26" s="8">
+        <f>$J$6 *$O$13 / $L$6</f>
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="27" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E27" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="F27" s="7">
+        <f>$J$6 / $O$14 / $K$6</f>
+        <v>62500</v>
+      </c>
+      <c r="G27" s="7">
+        <f>$J$6 / $O$14 / $L$6</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="28" spans="5:7" x14ac:dyDescent="0.3">
+      <c r="E28" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="F28" s="11">
+        <f>$J$6 / $O$15 / $K$6</f>
+        <v>31250</v>
+      </c>
+      <c r="G28" s="11">
+        <f>$J$6 / $O$15 / $L$6</f>
+        <v>500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Finish Implementing For Simple PWM
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_designHRTIM\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15595E55-9134-45ED-9550-FDC200154CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3B7FA5-8767-4266-90E0-EFF7327CB32E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="455">
   <si>
     <t>Colonne1</t>
   </si>
@@ -1550,7 +1550,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="8">
     <dxf>
       <font>
         <b val="0"/>
@@ -1709,9 +1709,6 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4358,20 +4355,6 @@
 </file>
 
 <file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{9E5B015E-0B8D-49DB-8A74-4F6D1452471D}" name="Tableau20" displayName="Tableau20" ref="E7:G15" totalsRowShown="0">
-  <autoFilter ref="E7:G15" xr:uid="{9E5B015E-0B8D-49DB-8A74-4F6D1452471D}"/>
-  <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{094F0F32-9797-4DD4-934E-F3C2C577DF5D}" name="Prescaler Ratio"/>
-    <tableColumn id="2" xr3:uid="{7661070E-E3D3-4CB7-B8A8-67A52F24F99B}" name="Min" dataDxfId="8">
-      <calculatedColumnFormula>$J$6 *$O$8 / $K$6</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{AF4C7D4D-6C03-4435-85F8-25E20A9543BE}" name="Max"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{234B95CE-5663-49A6-97EA-930C7F4E968E}" name="Tableau21" displayName="Tableau21" ref="E20:G28" totalsRowShown="0" headerRowDxfId="7" dataDxfId="5" headerRowBorderDxfId="6" tableBorderDxfId="4" totalsRowBorderDxfId="3">
   <autoFilter ref="E20:G28" xr:uid="{234B95CE-5663-49A6-97EA-930C7F4E968E}"/>
   <tableColumns count="3">
@@ -15452,109 +15435,42 @@
         <v>64000</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="E7" t="s">
-        <v>449</v>
-      </c>
-      <c r="F7" t="s">
-        <v>450</v>
-      </c>
-      <c r="G7" t="s">
-        <v>451</v>
-      </c>
-    </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="E8" t="s">
-        <v>441</v>
-      </c>
-      <c r="F8">
-        <f t="shared" ref="F8:F15" si="0">$J$6 *$O$8 / $K$6</f>
-        <v>4000000</v>
-      </c>
       <c r="O8">
         <v>32</v>
       </c>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="E9" t="s">
-        <v>442</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="0"/>
-        <v>4000000</v>
-      </c>
       <c r="O9">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="E10" t="s">
-        <v>443</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="0"/>
-        <v>4000000</v>
-      </c>
       <c r="O10">
         <v>8</v>
       </c>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="E11" t="s">
-        <v>444</v>
-      </c>
-      <c r="F11">
-        <f t="shared" si="0"/>
-        <v>4000000</v>
-      </c>
       <c r="O11">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="E12" t="s">
-        <v>445</v>
-      </c>
-      <c r="F12">
-        <f t="shared" si="0"/>
-        <v>4000000</v>
-      </c>
       <c r="O12">
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="E13" t="s">
-        <v>446</v>
-      </c>
-      <c r="F13">
-        <f t="shared" si="0"/>
-        <v>4000000</v>
-      </c>
       <c r="O13">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="E14" t="s">
-        <v>447</v>
-      </c>
-      <c r="F14">
-        <f t="shared" si="0"/>
-        <v>4000000</v>
-      </c>
       <c r="O14">
         <v>2</v>
       </c>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="E15" t="s">
-        <v>448</v>
-      </c>
-      <c r="F15">
-        <f t="shared" si="0"/>
-        <v>4000000</v>
-      </c>
       <c r="O15">
         <v>4</v>
       </c>
@@ -15676,9 +15592,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="2">
+  <tableParts count="1">
     <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
code gen for FMKHRT
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_designHRTIM\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97331EB3-762D-4DBF-B000-730BFE77A53B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84DB073-DCE4-41FB-B482-1AF0847BB781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
     <sheet name="FMK_IO" sheetId="2" r:id="rId2"/>
     <sheet name="FMK_TIM" sheetId="3" r:id="rId3"/>
-    <sheet name="FMK_CDA" sheetId="4" r:id="rId4"/>
-    <sheet name="FMKMAC" sheetId="6" r:id="rId5"/>
-    <sheet name="FMKCAN" sheetId="7" r:id="rId6"/>
-    <sheet name="FMKSRL" sheetId="8" r:id="rId7"/>
-    <sheet name="Feuil1" sheetId="5" r:id="rId8"/>
-    <sheet name="HRTIM_FreqHelp" sheetId="9" r:id="rId9"/>
+    <sheet name="FMKHRT" sheetId="10" r:id="rId4"/>
+    <sheet name="FMK_CDA" sheetId="4" r:id="rId5"/>
+    <sheet name="FMKMAC" sheetId="6" r:id="rId6"/>
+    <sheet name="FMKCAN" sheetId="7" r:id="rId7"/>
+    <sheet name="FMKSRL" sheetId="8" r:id="rId8"/>
+    <sheet name="Feuil1" sheetId="5" r:id="rId9"/>
+    <sheet name="HRTIM_FreqHelp" sheetId="9" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="470">
   <si>
     <t>Colonne1</t>
   </si>
@@ -1409,6 +1410,51 @@
   </si>
   <si>
     <t>Max ARR</t>
+  </si>
+  <si>
+    <t>HRTIM1_TIMD_IRQHandler</t>
+  </si>
+  <si>
+    <t>HRTIM1_TIMB_IRQHandler</t>
+  </si>
+  <si>
+    <t>HRTIM1_TIMA_IRQHandler</t>
+  </si>
+  <si>
+    <t>HRTIM1_TIMC_IRQHandler</t>
+  </si>
+  <si>
+    <t>HRTIM1_TIME_IRQHandler</t>
+  </si>
+  <si>
+    <t>HRTIM1_TIMF_IRQHandler</t>
+  </si>
+  <si>
+    <t>HRTIM1_Master_IRQHandler</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> HRTIM1_TIME_IRQHandler</t>
+  </si>
+  <si>
+    <t>Hrtimer name</t>
+  </si>
+  <si>
+    <t>nombre de Hrtim Index</t>
+  </si>
+  <si>
+    <t>nombre de channel par index</t>
+  </si>
+  <si>
+    <t>Timer Type</t>
+  </si>
+  <si>
+    <t>Tim</t>
+  </si>
+  <si>
+    <t>HrTim</t>
+  </si>
+  <si>
+    <t>TIMER_A</t>
   </si>
 </sst>
 </file>
@@ -4034,16 +4080,6 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{7B17A539-E635-4152-9412-9ADCB0D5ADE1}" name="Tableau26" displayName="Tableau26" ref="AF46:AF49" totalsRowShown="0">
-  <autoFilter ref="AF46:AF49" xr:uid="{7B17A539-E635-4152-9412-9ADCB0D5ADE1}"/>
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{41DEADB1-B8AC-4DA1-AAC6-1E2E0AF40D54}" name="Timer Purpose"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{00403EF2-391D-4DDF-AB62-FECA73965F51}" name="Tableau27" displayName="Tableau27" ref="A27:B30" totalsRowShown="0">
   <autoFilter ref="A27:B30" xr:uid="{00403EF2-391D-4DDF-AB62-FECA73965F51}"/>
   <tableColumns count="2">
@@ -4054,7 +4090,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="28" xr:uid="{93312290-37F4-462E-A13D-1DDA737E97BF}" name="GI_OSCILLATOR" displayName="GI_OSCILLATOR" ref="AF52:AF62" totalsRowShown="0">
   <autoFilter ref="AF52:AF62" xr:uid="{93312290-37F4-462E-A13D-1DDA737E97BF}"/>
   <tableColumns count="1">
@@ -4064,7 +4100,32 @@
 </table>
 </file>
 
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A27CADD5-26F4-4DF6-9D41-CEE02A85C4E9}" name="GI_ADC" displayName="GI_ADC" ref="V40:Y45" totalsRowShown="0">
+  <autoFilter ref="V40:Y45" xr:uid="{A27CADD5-26F4-4DF6-9D41-CEE02A85C4E9}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{46462DEE-B3A7-45AD-A2F8-63AC8C3C0154}" name="ADC_Name"/>
+    <tableColumn id="2" xr3:uid="{20DF5352-4B39-416D-A6E4-D94E56AED1C9}" name="number of channel"/>
+    <tableColumn id="3" xr3:uid="{9F9316C2-2066-47BF-B84E-436D4C41B07C}" name="IRQN assoiated"/>
+    <tableColumn id="4" xr3:uid="{CC116C4D-98B0-46BC-A882-0B90828FFD68}" name="Clock Associated"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{63985806-4671-4150-A59F-98E6B2C471BA}" name="GI_HrtilInfo" displayName="GI_HrtilInfo" ref="R17:T18" totalsRowShown="0">
+  <autoFilter ref="R17:T18" xr:uid="{63985806-4671-4150-A59F-98E6B2C471BA}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{87C5806D-8293-4916-B59E-5E76BE05E3ED}" name="Hrtimer name"/>
+    <tableColumn id="2" xr3:uid="{A78231C8-8605-4216-BF2D-099B66029CBE}" name="nombre de Hrtim Index"/>
+    <tableColumn id="3" xr3:uid="{604294EB-19ED-4821-9423-59CF7B6B156E}" name="nombre de channel par index"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}" name="FMKIO_InputDig" displayName="FMKIO_InputDig" ref="A6:B14" totalsRowShown="0">
   <autoFilter ref="A6:B14" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}"/>
   <tableColumns count="2">
@@ -4075,9 +4136,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}" name="FMKIO_OutputDig" displayName="FMKIO_OutputDig" ref="Z7:AA16" totalsRowShown="0">
-  <autoFilter ref="Z7:AA16" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}"/>
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}" name="FMKIO_OutputDig" displayName="FMKIO_OutputDig" ref="AA7:AB16" totalsRowShown="0">
+  <autoFilter ref="AA7:AB16" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{395BD36A-0840-48CF-8D8D-56878E366FC5}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{34DF2CF3-8826-4F9E-A09D-280EE0FEFFBB}" name="Pin_name"/>
@@ -4086,7 +4147,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{27D0C574-E325-48F5-AA31-7FBAF1E09007}" name="FMKIO_InputFreq" displayName="FMKIO_InputFreq" ref="J6:N10" totalsRowShown="0">
   <autoFilter ref="J6:N10" xr:uid="{27D0C574-E325-48F5-AA31-7FBAF1E09007}"/>
   <tableColumns count="5">
@@ -4100,9 +4161,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}" name="FMKIO_InputEvnt" displayName="FMKIO_InputEvnt" ref="V6:X8" totalsRowShown="0">
-  <autoFilter ref="V6:X8" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}"/>
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}" name="FMKIO_InputEvnt" displayName="FMKIO_InputEvnt" ref="W6:Y8" totalsRowShown="0">
+  <autoFilter ref="W6:Y8" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5C8A98A4-9028-4F61-A263-67D85D1BFF84}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{D3F2DFB4-9CF8-4086-ABAA-63BD13D3A4C5}" name="Pin_name"/>
@@ -4112,21 +4173,22 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{DE41CD30-BCBD-40FE-B5DD-848DAAA9C25B}" name="FMKIO_OutputPwm" displayName="FMKIO_OutputPwm" ref="P6:T18" totalsRowShown="0">
-  <autoFilter ref="P6:T18" xr:uid="{DE41CD30-BCBD-40FE-B5DD-848DAAA9C25B}"/>
-  <tableColumns count="5">
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{DE41CD30-BCBD-40FE-B5DD-848DAAA9C25B}" name="FMKIO_OutputPwm" displayName="FMKIO_OutputPwm" ref="P6:U18" totalsRowShown="0">
+  <autoFilter ref="P6:U18" xr:uid="{DE41CD30-BCBD-40FE-B5DD-848DAAA9C25B}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{F2B685DB-87AE-429A-9E70-076DA856F9A2}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{30126296-E33C-4D56-9110-2D49FE159CF1}" name="Pin_name"/>
     <tableColumn id="3" xr3:uid="{40FECABF-BB72-44BD-85CF-471C0A6DFCAD}" name="alternate function timer"/>
     <tableColumn id="4" xr3:uid="{B11B3F8E-B4EB-4DA0-9576-7D8704B7B2D1}" name="Timer "/>
     <tableColumn id="5" xr3:uid="{7FD00E0A-7E1B-4877-A449-DCC379CE738A}" name="Timer_channel"/>
+    <tableColumn id="6" xr3:uid="{9AFC2953-12BB-4E45-95D4-96A745007A18}" name="Timer Type"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}" name="FMKIO_InputAna" displayName="FMKIO_InputAna" ref="E6:H11" totalsRowShown="0">
   <autoFilter ref="E6:H11" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}"/>
   <tableColumns count="4">
@@ -4134,16 +4196,6 @@
     <tableColumn id="2" xr3:uid="{75AD9B1E-8F88-4CD9-86AB-C0D6BFDB44CD}" name="Pin_name"/>
     <tableColumn id="3" xr3:uid="{1D048BA7-3BEB-4D49-9106-38D6D8BF0832}" name="ADC_Used"/>
     <tableColumn id="4" xr3:uid="{2343B7ED-C668-4AE0-9949-C8D70A9AC2BF}" name="Adc_Channel"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{3EEFA786-828B-422C-9405-D0B0DD120CF4}" name="Tableau17" displayName="Tableau17" ref="AW29:AW45" totalsRowShown="0">
-  <autoFilter ref="AW29:AW45" xr:uid="{3EEFA786-828B-422C-9405-D0B0DD120CF4}"/>
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{01BF5210-733A-4DB1-A72E-FC1B749F7F18}" name="Pin_Choice"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4161,6 +4213,16 @@
 </file>
 
 <file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{3EEFA786-828B-422C-9405-D0B0DD120CF4}" name="Tableau17" displayName="Tableau17" ref="AW29:AW45" totalsRowShown="0">
+  <autoFilter ref="AW29:AW45" xr:uid="{3EEFA786-828B-422C-9405-D0B0DD120CF4}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{01BF5210-733A-4DB1-A72E-FC1B749F7F18}" name="Pin_Choice"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{06E0084F-32F1-4C7D-A6E0-EE7152DB4CBF}" name="Tableau18" displayName="Tableau18" ref="AY30:AY34" totalsRowShown="0">
   <autoFilter ref="AY30:AY34" xr:uid="{06E0084F-32F1-4C7D-A6E0-EE7152DB4CBF}"/>
   <tableColumns count="1">
@@ -4170,7 +4232,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{9F1C0A09-0E71-42DD-A451-D3B53F431EBF}" name="Tableau1720" displayName="Tableau1720" ref="BA29:BA47" totalsRowShown="0">
   <autoFilter ref="BA29:BA47" xr:uid="{9F1C0A09-0E71-42DD-A451-D3B53F431EBF}"/>
   <tableColumns count="1">
@@ -4180,7 +4242,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{0413BBED-76B8-4200-A43C-D97EFAA1EA94}" name="FMKIO_CanCfg" displayName="FMKIO_CanCfg" ref="A25:F28" totalsRowShown="0">
   <autoFilter ref="A25:F28" xr:uid="{0413BBED-76B8-4200-A43C-D97EFAA1EA94}"/>
   <tableColumns count="6">
@@ -4195,7 +4257,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{978057A4-13F6-44F3-B65B-2C409866E1DE}" name="FMKIO_SerialCfg" displayName="FMKIO_SerialCfg" ref="A34:F36" totalsRowShown="0">
   <autoFilter ref="A34:F36" xr:uid="{978057A4-13F6-44F3-B65B-2C409866E1DE}"/>
   <tableColumns count="6">
@@ -4210,7 +4272,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{DA1831B2-BC94-42A9-B299-31A3CE618396}" name="FMKIO_IRQNHandler" displayName="FMKIO_IRQNHandler" ref="W29:W36" totalsRowShown="0">
   <autoFilter ref="W29:W36" xr:uid="{DA1831B2-BC94-42A9-B299-31A3CE618396}"/>
   <tableColumns count="1">
@@ -4220,7 +4282,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{684AB3A4-4693-477C-AADC-64EBB335C3E9}" name="FMKTIM_EvntTimer" displayName="FMKTIM_EvntTimer" ref="B4:C6" totalsRowShown="0">
   <autoFilter ref="B4:C6" xr:uid="{684AB3A4-4693-477C-AADC-64EBB335C3E9}"/>
   <tableColumns count="2">
@@ -4231,7 +4293,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{CCB68487-82CB-434C-A0E4-701B1FDDACF5}" name="FMKTIM_IRQNHandler" displayName="FMKTIM_IRQNHandler" ref="F4:G17" totalsRowShown="0">
   <autoFilter ref="F4:G17" xr:uid="{CCB68487-82CB-434C-A0E4-701B1FDDACF5}"/>
   <tableColumns count="2">
@@ -4242,7 +4304,17 @@
 </table>
 </file>
 
-<file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{953E7E02-522E-4F1F-B136-4D0BF069F045}" name="FMKHRT_IrqHandler" displayName="FMKHRT_IrqHandler" ref="Y5:Y13" totalsRowShown="0">
+  <autoFilter ref="Y5:Y13" xr:uid="{953E7E02-522E-4F1F-B136-4D0BF069F045}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{4F3F9E81-1A81-491D-8B79-C106AA82CA37}" name="Colonne1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{A4F27ADC-56A6-479B-93EF-D6AA72368D72}" name="FMKCDA_CalibrationOthers" displayName="FMKCDA_CalibrationOthers" ref="I3:L5" totalsRowShown="0">
   <autoFilter ref="I3:L5" xr:uid="{A4F27ADC-56A6-479B-93EF-D6AA72368D72}"/>
   <tableColumns count="4">
@@ -4255,7 +4327,18 @@
 </table>
 </file>
 
-<file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5A8C957F-EDE6-44F1-B8F8-2086E255196A}" name="GI_DAC" displayName="GI_DAC" ref="Y36:Z37" totalsRowShown="0">
+  <autoFilter ref="Y36:Z37" xr:uid="{5A8C957F-EDE6-44F1-B8F8-2086E255196A}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{73150C50-6B2A-4CD8-A7E6-62C171935AF8}" name="DAC_Name"/>
+    <tableColumn id="2" xr3:uid="{EF9B5413-9A3C-4163-8063-C74DAB2D51F7}" name="number of channel"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}" name="FMKCDA_VoltageRef" displayName="FMKCDA_VoltageRef" ref="S3:V8" totalsRowShown="0">
   <autoFilter ref="S3:V8" xr:uid="{99B4503A-67B2-48AD-BE25-2B3425F892A9}"/>
   <tableColumns count="4">
@@ -4268,7 +4351,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="33" xr:uid="{FAF38277-E25D-413A-A145-AFBC74566FF1}" name="FMKCDA_IRQNHandler" displayName="FMKCDA_IRQNHandler" ref="E8:F12" totalsRowShown="0">
   <autoFilter ref="E8:F12" xr:uid="{FAF38277-E25D-413A-A145-AFBC74566FF1}"/>
   <tableColumns count="2">
@@ -4279,20 +4362,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A27CADD5-26F4-4DF6-9D41-CEE02A85C4E9}" name="GI_ADC" displayName="GI_ADC" ref="T20:W25" totalsRowShown="0">
-  <autoFilter ref="T20:W25" xr:uid="{A27CADD5-26F4-4DF6-9D41-CEE02A85C4E9}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{46462DEE-B3A7-45AD-A2F8-63AC8C3C0154}" name="ADC_Name"/>
-    <tableColumn id="2" xr3:uid="{20DF5352-4B39-416D-A6E4-D94E56AED1C9}" name="number of channel"/>
-    <tableColumn id="3" xr3:uid="{9F9316C2-2066-47BF-B84E-436D4C41B07C}" name="IRQN assoiated"/>
-    <tableColumn id="4" xr3:uid="{CC116C4D-98B0-46BC-A882-0B90828FFD68}" name="Clock Associated"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}" name="FMKMAC_Cfg" displayName="FMKMAC_Cfg" ref="B2:E12" totalsRowShown="0">
   <autoFilter ref="B2:E12" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}"/>
   <tableColumns count="4">
@@ -4305,7 +4375,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="34" xr:uid="{8B613F4D-88F2-4091-AA3A-5550AB627653}" name="FMKMAC_IRQN" displayName="FMKMAC_IRQN" ref="J3:K18" totalsRowShown="0">
   <autoFilter ref="J3:K18" xr:uid="{8B613F4D-88F2-4091-AA3A-5550AB627653}"/>
   <tableColumns count="2">
@@ -4316,7 +4386,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="36" xr:uid="{9E75F4B3-8C66-44CB-A927-82E8A09563A2}" name="FMKMAC_DMAMUX" displayName="FMKMAC_DMAMUX" ref="P3:P4" totalsRowShown="0">
   <autoFilter ref="P3:P4" xr:uid="{9E75F4B3-8C66-44CB-A927-82E8A09563A2}"/>
   <tableColumns count="1">
@@ -4326,7 +4396,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{3568793B-2270-4B9A-A9E5-55F929444AFF}" name="Tableau35" displayName="Tableau35" ref="B5:B11" totalsRowShown="0">
   <autoFilter ref="B5:B11" xr:uid="{3568793B-2270-4B9A-A9E5-55F929444AFF}"/>
   <tableColumns count="1">
@@ -4336,7 +4406,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table36.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="37" xr:uid="{CF6032E9-4D15-4575-AD94-133BB9C2FD31}" name="FMKSRL_INFO" displayName="FMKSRL_INFO" ref="E2:M7" totalsRowShown="0">
   <autoFilter ref="E2:M7" xr:uid="{CF6032E9-4D15-4575-AD94-133BB9C2FD31}"/>
   <tableColumns count="9">
@@ -4354,7 +4424,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table37.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{234B95CE-5663-49A6-97EA-930C7F4E968E}" name="Tableau21" displayName="Tableau21" ref="E20:G28" totalsRowShown="0" headerRowDxfId="7" dataDxfId="5" headerRowBorderDxfId="6" tableBorderDxfId="4" totalsRowBorderDxfId="3">
   <autoFilter ref="E20:G28" xr:uid="{234B95CE-5663-49A6-97EA-930C7F4E968E}"/>
   <tableColumns count="3">
@@ -4367,17 +4437,6 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5A8C957F-EDE6-44F1-B8F8-2086E255196A}" name="GI_DAC" displayName="GI_DAC" ref="Y36:Z37" totalsRowShown="0">
-  <autoFilter ref="Y36:Z37" xr:uid="{5A8C957F-EDE6-44F1-B8F8-2086E255196A}"/>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{73150C50-6B2A-4CD8-A7E6-62C171935AF8}" name="DAC_Name"/>
-    <tableColumn id="2" xr3:uid="{EF9B5413-9A3C-4163-8063-C74DAB2D51F7}" name="number of channel"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0BD818BF-294B-4FA2-8E5A-7FD1DB70B357}" name="GI_IRQN" displayName="GI_IRQN" ref="H18:I119" totalsRowShown="0">
   <autoFilter ref="H18:I119" xr:uid="{0BD818BF-294B-4FA2-8E5A-7FD1DB70B357}"/>
   <tableColumns count="2">
@@ -4388,7 +4447,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9B4F1398-0B6D-4B55-A4C3-611E0B66A012}" name="GI_RCC_CLOCK" displayName="GI_RCC_CLOCK" ref="D18:F75" totalsRowShown="0">
   <autoFilter ref="D18:F75" xr:uid="{9B4F1398-0B6D-4B55-A4C3-611E0B66A012}"/>
   <tableColumns count="3">
@@ -4400,7 +4459,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FC2F87AB-FFF7-4006-99CC-8D938E27338D}" name="GI_DMA" displayName="GI_DMA" ref="AB20:AD22" totalsRowShown="0">
   <autoFilter ref="AB20:AD22" xr:uid="{FC2F87AB-FFF7-4006-99CC-8D938E27338D}"/>
   <tableColumns count="3">
@@ -4412,7 +4471,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{13E9277E-229F-41F0-9B99-7D1A0B71D1B3}" name="Tableau16" displayName="Tableau16" ref="AF40:AF43" totalsRowShown="0">
   <autoFilter ref="AF40:AF43" xr:uid="{13E9277E-229F-41F0-9B99-7D1A0B71D1B3}"/>
   <tableColumns count="1">
@@ -4422,11 +4481,21 @@
 </table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{69B16F87-38FA-4931-845E-91EC8B0FFB29}" name="CPU_Config" displayName="CPU_Config" ref="B18:B19" totalsRowShown="0">
   <autoFilter ref="B18:B19" xr:uid="{69B16F87-38FA-4931-845E-91EC8B0FFB29}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{FD4FECA3-1A39-43C0-8443-3217FDF815FF}" name="STM32 Processor "/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{7B17A539-E635-4152-9412-9ADCB0D5ADE1}" name="Tableau26" displayName="Tableau26" ref="AF46:AF49" totalsRowShown="0">
+  <autoFilter ref="AF46:AF49" xr:uid="{7B17A539-E635-4152-9412-9ADCB0D5ADE1}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{41DEADB1-B8AC-4DA1-AAC6-1E2E0AF40D54}" name="Timer Purpose"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4749,7 +4818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{871E2D6D-43F7-44B1-8255-ECFDDA33AA9C}">
-  <dimension ref="A18:AF119"/>
+  <dimension ref="A17:AF119"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.6640625" customWidth="1"/>
@@ -4767,7 +4836,9 @@
     <col min="15" max="15" width="22.77734375" customWidth="1"/>
     <col min="16" max="16" width="23.44140625" customWidth="1"/>
     <col min="17" max="17" width="20.6640625" customWidth="1"/>
-    <col min="20" max="20" width="21.33203125" customWidth="1"/>
+    <col min="18" max="18" width="21" customWidth="1"/>
+    <col min="19" max="19" width="33.88671875" customWidth="1"/>
+    <col min="20" max="20" width="35.33203125" customWidth="1"/>
     <col min="21" max="21" width="21.21875" customWidth="1"/>
     <col min="22" max="22" width="19.109375" customWidth="1"/>
     <col min="23" max="23" width="18.77734375" customWidth="1"/>
@@ -4776,6 +4847,17 @@
     <col min="31" max="31" width="17.77734375" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="R17" t="s">
+        <v>463</v>
+      </c>
+      <c r="S17" t="s">
+        <v>464</v>
+      </c>
+      <c r="T17" t="s">
+        <v>465</v>
+      </c>
+    </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>122</v>
@@ -4810,6 +4892,15 @@
       <c r="O18" t="s">
         <v>296</v>
       </c>
+      <c r="R18" t="s">
+        <v>250</v>
+      </c>
+      <c r="S18">
+        <v>6</v>
+      </c>
+      <c r="T18">
+        <v>2</v>
+      </c>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
@@ -4877,18 +4968,6 @@
       <c r="O20" t="s">
         <v>294</v>
       </c>
-      <c r="T20" t="s">
-        <v>17</v>
-      </c>
-      <c r="U20" t="s">
-        <v>18</v>
-      </c>
-      <c r="V20" t="s">
-        <v>275</v>
-      </c>
-      <c r="W20" t="s">
-        <v>276</v>
-      </c>
       <c r="AB20" t="s">
         <v>22</v>
       </c>
@@ -4930,18 +5009,6 @@
       <c r="O21" t="s">
         <v>294</v>
       </c>
-      <c r="T21" t="s">
-        <v>16</v>
-      </c>
-      <c r="U21">
-        <v>18</v>
-      </c>
-      <c r="V21" t="s">
-        <v>138</v>
-      </c>
-      <c r="W21" t="s">
-        <v>237</v>
-      </c>
       <c r="AB21" t="s">
         <v>331</v>
       </c>
@@ -4983,18 +5050,6 @@
       <c r="O22" t="s">
         <v>294</v>
       </c>
-      <c r="T22" t="s">
-        <v>261</v>
-      </c>
-      <c r="U22">
-        <v>18</v>
-      </c>
-      <c r="V22" t="s">
-        <v>138</v>
-      </c>
-      <c r="W22" t="s">
-        <v>237</v>
-      </c>
       <c r="AB22" t="s">
         <v>332</v>
       </c>
@@ -5036,18 +5091,6 @@
       <c r="O23" t="s">
         <v>294</v>
       </c>
-      <c r="T23" t="s">
-        <v>262</v>
-      </c>
-      <c r="U23">
-        <v>18</v>
-      </c>
-      <c r="V23" t="s">
-        <v>161</v>
-      </c>
-      <c r="W23" t="s">
-        <v>238</v>
-      </c>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="D24" t="s">
@@ -5080,18 +5123,6 @@
       <c r="O24" t="s">
         <v>294</v>
       </c>
-      <c r="T24" t="s">
-        <v>263</v>
-      </c>
-      <c r="U24">
-        <v>18</v>
-      </c>
-      <c r="V24" t="s">
-        <v>175</v>
-      </c>
-      <c r="W24" t="s">
-        <v>238</v>
-      </c>
     </row>
     <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="D25" t="s">
@@ -5124,18 +5155,6 @@
       <c r="O25" t="s">
         <v>295</v>
       </c>
-      <c r="T25" t="s">
-        <v>264</v>
-      </c>
-      <c r="U25">
-        <v>18</v>
-      </c>
-      <c r="V25" t="s">
-        <v>176</v>
-      </c>
-      <c r="W25" t="s">
-        <v>238</v>
-      </c>
     </row>
     <row r="26" spans="1:30" x14ac:dyDescent="0.3">
       <c r="D26" t="s">
@@ -5544,6 +5563,18 @@
       <c r="Q40">
         <v>11</v>
       </c>
+      <c r="V40" t="s">
+        <v>17</v>
+      </c>
+      <c r="W40" t="s">
+        <v>18</v>
+      </c>
+      <c r="X40" t="s">
+        <v>275</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>276</v>
+      </c>
       <c r="AF40" t="s">
         <v>88</v>
       </c>
@@ -5564,6 +5595,18 @@
       <c r="I41" t="s">
         <v>90</v>
       </c>
+      <c r="V41" t="s">
+        <v>16</v>
+      </c>
+      <c r="W41">
+        <v>18</v>
+      </c>
+      <c r="X41" t="s">
+        <v>138</v>
+      </c>
+      <c r="Y41" t="s">
+        <v>237</v>
+      </c>
       <c r="AF41" t="s">
         <v>89</v>
       </c>
@@ -5584,6 +5627,18 @@
       <c r="I42" t="s">
         <v>69</v>
       </c>
+      <c r="V42" t="s">
+        <v>261</v>
+      </c>
+      <c r="W42">
+        <v>18</v>
+      </c>
+      <c r="X42" t="s">
+        <v>138</v>
+      </c>
+      <c r="Y42" t="s">
+        <v>237</v>
+      </c>
       <c r="AF42" t="s">
         <v>69</v>
       </c>
@@ -5604,6 +5659,18 @@
       <c r="I43" t="s">
         <v>69</v>
       </c>
+      <c r="V43" t="s">
+        <v>262</v>
+      </c>
+      <c r="W43">
+        <v>18</v>
+      </c>
+      <c r="X43" t="s">
+        <v>161</v>
+      </c>
+      <c r="Y43" t="s">
+        <v>238</v>
+      </c>
       <c r="AF43" t="s">
         <v>90</v>
       </c>
@@ -5624,6 +5691,18 @@
       <c r="I44" t="s">
         <v>69</v>
       </c>
+      <c r="V44" t="s">
+        <v>263</v>
+      </c>
+      <c r="W44">
+        <v>18</v>
+      </c>
+      <c r="X44" t="s">
+        <v>175</v>
+      </c>
+      <c r="Y44" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="45" spans="4:32" x14ac:dyDescent="0.3">
       <c r="D45" t="s">
@@ -5640,6 +5719,18 @@
       </c>
       <c r="I45" t="s">
         <v>69</v>
+      </c>
+      <c r="V45" t="s">
+        <v>264</v>
+      </c>
+      <c r="W45">
+        <v>18</v>
+      </c>
+      <c r="X45" t="s">
+        <v>176</v>
+      </c>
+      <c r="Y45" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="46" spans="4:32" x14ac:dyDescent="0.3">
@@ -6567,7 +6658,7 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <tableParts count="12">
+  <tableParts count="13">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
@@ -6580,6 +6671,209 @@
     <tablePart r:id="rId11"/>
     <tablePart r:id="rId12"/>
     <tablePart r:id="rId13"/>
+    <tablePart r:id="rId14"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34ECC9F7-B649-41BF-A742-3CCEA0266A56}">
+  <dimension ref="B3:R28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="18.77734375" customWidth="1"/>
+    <col min="6" max="6" width="20.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:15" ht="93.6" x14ac:dyDescent="1.75">
+      <c r="B3" s="6" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="J5" t="s">
+        <v>452</v>
+      </c>
+      <c r="K5" t="s">
+        <v>453</v>
+      </c>
+      <c r="L5" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="J6">
+        <v>128000000</v>
+      </c>
+      <c r="K6">
+        <v>1024</v>
+      </c>
+      <c r="L6">
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="O8">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="O9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="O10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="O11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="O12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="O13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="O14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="O15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="5:18" x14ac:dyDescent="0.3">
+      <c r="E20" s="9" t="s">
+        <v>449</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="21" spans="5:18" x14ac:dyDescent="0.3">
+      <c r="E21" s="7" t="s">
+        <v>441</v>
+      </c>
+      <c r="F21" s="7">
+        <f>$J$6 *$O$8 / $K$6</f>
+        <v>4000000</v>
+      </c>
+      <c r="G21" s="7">
+        <f>$J$6 *$O$8 / $L$6</f>
+        <v>64000</v>
+      </c>
+    </row>
+    <row r="22" spans="5:18" x14ac:dyDescent="0.3">
+      <c r="E22" s="8" t="s">
+        <v>442</v>
+      </c>
+      <c r="F22" s="8">
+        <f>$J$6 *$O$9 / $K$6</f>
+        <v>2000000</v>
+      </c>
+      <c r="G22" s="8">
+        <f>$J$6 *$O$9 / $L$6</f>
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="23" spans="5:18" x14ac:dyDescent="0.3">
+      <c r="E23" s="7" t="s">
+        <v>443</v>
+      </c>
+      <c r="F23" s="7">
+        <f>$J$6 *$O$10 / $K$6</f>
+        <v>1000000</v>
+      </c>
+      <c r="G23" s="7">
+        <f>$J$6 *$O$10 / $L$6</f>
+        <v>16000</v>
+      </c>
+      <c r="R23" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="5:18" x14ac:dyDescent="0.3">
+      <c r="E24" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="F24" s="8">
+        <f>$J$6 *$O$11 / $K$6</f>
+        <v>500000</v>
+      </c>
+      <c r="G24" s="8">
+        <f>$J$6 *$O$11 / $L$6</f>
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="25" spans="5:18" x14ac:dyDescent="0.3">
+      <c r="E25" s="7" t="s">
+        <v>445</v>
+      </c>
+      <c r="F25" s="7">
+        <f>$J$6 *$O$12 / $K$6</f>
+        <v>250000</v>
+      </c>
+      <c r="G25" s="7">
+        <f>$J$6 *$O$12 / $L$6</f>
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="26" spans="5:18" x14ac:dyDescent="0.3">
+      <c r="E26" s="8" t="s">
+        <v>446</v>
+      </c>
+      <c r="F26" s="8">
+        <f>$J$6 *$O$13 / $K$6</f>
+        <v>125000</v>
+      </c>
+      <c r="G26" s="8">
+        <f>$J$6 *$O$13 / $L$6</f>
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="27" spans="5:18" x14ac:dyDescent="0.3">
+      <c r="E27" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="F27" s="7">
+        <f>$J$6 / $O$14 / $K$6</f>
+        <v>62500</v>
+      </c>
+      <c r="G27" s="7">
+        <f>$J$6 / $O$14 / $L$6</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="28" spans="5:18" x14ac:dyDescent="0.3">
+      <c r="E28" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="F28" s="11">
+        <f>$J$6 / $O$15 / $K$6</f>
+        <v>31250</v>
+      </c>
+      <c r="G28" s="11">
+        <f>$J$6 / $O$15 / $L$6</f>
+        <v>500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6617,7 +6911,7 @@
     <col min="40" max="40" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>439</v>
       </c>
@@ -6625,7 +6919,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -6648,7 +6942,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -6697,20 +6991,23 @@
       <c r="T6" t="s">
         <v>44</v>
       </c>
-      <c r="V6" t="s">
+      <c r="U6" t="s">
+        <v>466</v>
+      </c>
+      <c r="W6" t="s">
         <v>23</v>
       </c>
-      <c r="W6" t="s">
+      <c r="X6" t="s">
         <v>24</v>
       </c>
-      <c r="X6" t="s">
+      <c r="Y6" t="s">
         <v>47</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AA6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6759,23 +7056,26 @@
       <c r="T7" t="s">
         <v>46</v>
       </c>
-      <c r="V7" t="s">
+      <c r="U7" t="s">
+        <v>467</v>
+      </c>
+      <c r="W7" t="s">
         <v>12</v>
       </c>
-      <c r="W7" t="s">
+      <c r="X7" t="s">
         <v>27</v>
       </c>
-      <c r="X7" t="s">
+      <c r="Y7" t="s">
         <v>435</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AA7" t="s">
         <v>23</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="AB7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -6824,23 +7124,26 @@
       <c r="T8" t="s">
         <v>92</v>
       </c>
-      <c r="V8" t="s">
+      <c r="U8" t="s">
+        <v>467</v>
+      </c>
+      <c r="W8" t="s">
         <v>12</v>
       </c>
-      <c r="W8" t="s">
+      <c r="X8" t="s">
         <v>30</v>
       </c>
-      <c r="X8" t="s">
+      <c r="Y8" t="s">
         <v>436</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="AA8" t="s">
         <v>12</v>
       </c>
-      <c r="AA8" t="s">
+      <c r="AB8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -6889,14 +7192,17 @@
       <c r="T9" t="s">
         <v>46</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="U9" t="s">
+        <v>467</v>
+      </c>
+      <c r="AA9" t="s">
         <v>12</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AB9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -6945,14 +7251,17 @@
       <c r="T10" t="s">
         <v>50</v>
       </c>
-      <c r="Z10" t="s">
+      <c r="U10" t="s">
+        <v>467</v>
+      </c>
+      <c r="AA10" t="s">
         <v>12</v>
       </c>
-      <c r="AA10" t="s">
+      <c r="AB10" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -6986,14 +7295,17 @@
       <c r="T11" t="s">
         <v>45</v>
       </c>
-      <c r="Z11" t="s">
+      <c r="U11" t="s">
+        <v>467</v>
+      </c>
+      <c r="AA11" t="s">
         <v>12</v>
       </c>
-      <c r="AA11" t="s">
+      <c r="AB11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -7015,14 +7327,17 @@
       <c r="T12" t="s">
         <v>46</v>
       </c>
-      <c r="Z12" t="s">
+      <c r="U12" t="s">
+        <v>467</v>
+      </c>
+      <c r="AA12" t="s">
         <v>12</v>
       </c>
-      <c r="AA12" t="s">
+      <c r="AB12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -7044,14 +7359,17 @@
       <c r="T13" t="s">
         <v>92</v>
       </c>
-      <c r="Z13" t="s">
+      <c r="U13" t="s">
+        <v>467</v>
+      </c>
+      <c r="AA13" t="s">
         <v>11</v>
       </c>
-      <c r="AA13" t="s">
+      <c r="AB13" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -7073,14 +7391,17 @@
       <c r="T14" t="s">
         <v>50</v>
       </c>
-      <c r="Z14" t="s">
+      <c r="U14" t="s">
+        <v>467</v>
+      </c>
+      <c r="AA14" t="s">
         <v>11</v>
       </c>
-      <c r="AA14" t="s">
+      <c r="AB14" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
       <c r="P15" t="s">
         <v>12</v>
       </c>
@@ -7096,14 +7417,17 @@
       <c r="T15" t="s">
         <v>45</v>
       </c>
-      <c r="Z15" t="s">
+      <c r="U15" t="s">
+        <v>467</v>
+      </c>
+      <c r="AA15" t="s">
         <v>11</v>
       </c>
-      <c r="AA15" t="s">
+      <c r="AB15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
       <c r="P16" t="s">
         <v>12</v>
       </c>
@@ -7119,10 +7443,13 @@
       <c r="T16" t="s">
         <v>46</v>
       </c>
-      <c r="Z16" t="s">
+      <c r="U16" t="s">
+        <v>467</v>
+      </c>
+      <c r="AA16" t="s">
         <v>14</v>
       </c>
-      <c r="AA16" t="s">
+      <c r="AB16" t="s">
         <v>27</v>
       </c>
     </row>
@@ -7137,10 +7464,13 @@
         <v>433</v>
       </c>
       <c r="S17" t="s">
-        <v>252</v>
+        <v>469</v>
       </c>
       <c r="T17" t="s">
-        <v>92</v>
+        <v>45</v>
+      </c>
+      <c r="U17" t="s">
+        <v>468</v>
       </c>
     </row>
     <row r="18" spans="1:53" x14ac:dyDescent="0.3">
@@ -7159,6 +7489,9 @@
       <c r="T18" t="s">
         <v>50</v>
       </c>
+      <c r="U18" t="s">
+        <v>467</v>
+      </c>
     </row>
     <row r="24" spans="1:53" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
@@ -7497,15 +7830,18 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 K7:K10 Q7:Q14 F7:F11 B7:B14 W7:W8 AA8:AA16" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 K7:K10 Q7:Q14 F7:F11 B7:B14 X7:X8 AB8:AB16" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
       <formula1>$AW$30:$AW$45</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T7:T14 N7:N10" xr:uid="{727A5344-B28A-4866-9EC1-7C96029AF8B6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N7:N10 T7:T14" xr:uid="{727A5344-B28A-4866-9EC1-7C96029AF8B6}">
       <formula1>$AY$31:$AY$34</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7:H11" xr:uid="{FFFA1AF2-B35F-4BAA-AEF6-4A6121806F8D}">
       <formula1>$BA$30:$BA$47</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U7:U20" xr:uid="{843CAB93-5FB8-4584-AA77-D87D9BF50E6D}">
+      <formula1>"HrTim,Tim"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7531,19 +7867,19 @@
           <x14:formula1>
             <xm:f>General_Info!$P$34:$P$39</xm:f>
           </x14:formula1>
-          <xm:sqref>P7:P14 J7:J10 E7:E11 A7:A14 V7:V8 Z8:Z16</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C428027-B16D-4B04-9CB2-8290577ED0FB}">
-          <x14:formula1>
-            <xm:f>General_Info!$T$21:$T$25</xm:f>
-          </x14:formula1>
-          <xm:sqref>G6:G11</xm:sqref>
+          <xm:sqref>P7:P14 J7:J10 E7:E11 A7:A14 W7:W8 AA8:AA16</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1C3D18C3-7241-4088-8034-07AAE0EB53A9}">
           <x14:formula1>
             <xm:f>General_Info!$K$19:$K$30</xm:f>
           </x14:formula1>
           <xm:sqref>S7:S14</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C428027-B16D-4B04-9CB2-8290577ED0FB}">
+          <x14:formula1>
+            <xm:f>General_Info!$V$41:$V$45</xm:f>
+          </x14:formula1>
+          <xm:sqref>G6:G11</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7711,6 +8047,67 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BF150CB-3330-4180-96AC-4A3D28CDB7F6}">
+  <dimension ref="Y5:Y13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="25" max="25" width="27.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="25:25" x14ac:dyDescent="0.3">
+      <c r="Y5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="25:25" x14ac:dyDescent="0.3">
+      <c r="Y6" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="7" spans="25:25" x14ac:dyDescent="0.3">
+      <c r="Y7" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="8" spans="25:25" x14ac:dyDescent="0.3">
+      <c r="Y8" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="9" spans="25:25" x14ac:dyDescent="0.3">
+      <c r="Y9" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="10" spans="25:25" x14ac:dyDescent="0.3">
+      <c r="Y10" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="11" spans="25:25" x14ac:dyDescent="0.3">
+      <c r="Y11" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="12" spans="25:25" x14ac:dyDescent="0.3">
+      <c r="Y12" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="13" spans="25:25" x14ac:dyDescent="0.3">
+      <c r="Y13" t="s">
+        <v>462</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0962FBCC-E1F3-44E3-92A8-D1FF17927B08}">
   <dimension ref="E2:V12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -7916,7 +8313,7 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9E258101-4BE3-4FFA-9159-E0120D35AA71}">
           <x14:formula1>
-            <xm:f>General_Info!$T$21:$T$25</xm:f>
+            <xm:f>General_Info!$V$41:$V$45</xm:f>
           </x14:formula1>
           <xm:sqref>K4:K5 U4:U8</xm:sqref>
         </x14:dataValidation>
@@ -7926,7 +8323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06E18236-E25D-41B3-8B1E-0194276152B3}">
   <dimension ref="B2:P18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -8208,7 +8605,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9D1D4C8-FD0D-4DBE-B311-5297C41CC83F}">
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -8266,7 +8663,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E85D06B3-E762-495B-BF06-A6CD7E704A4C}">
   <dimension ref="E2:M7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -8460,7 +8857,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{860CCB6B-9BC8-4B28-B4AE-B22F38F81573}">
   <dimension ref="B1:P254"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -15397,206 +15794,4 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34ECC9F7-B649-41BF-A742-3CCEA0266A56}">
-  <dimension ref="B3:R28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="5" max="5" width="18.77734375" customWidth="1"/>
-    <col min="6" max="6" width="20.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="2:15" ht="93.6" x14ac:dyDescent="1.75">
-      <c r="B3" s="6" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="J5" t="s">
-        <v>452</v>
-      </c>
-      <c r="K5" t="s">
-        <v>453</v>
-      </c>
-      <c r="L5" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="J6">
-        <v>128000000</v>
-      </c>
-      <c r="K6">
-        <v>1024</v>
-      </c>
-      <c r="L6">
-        <v>64000</v>
-      </c>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="O8">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="O9">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="O10">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="O11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="O12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="O13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="O14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="O15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="5:18" x14ac:dyDescent="0.3">
-      <c r="E20" s="9" t="s">
-        <v>449</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>451</v>
-      </c>
-      <c r="G20" s="10" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="21" spans="5:18" x14ac:dyDescent="0.3">
-      <c r="E21" s="7" t="s">
-        <v>441</v>
-      </c>
-      <c r="F21" s="7">
-        <f>$J$6 *$O$8 / $K$6</f>
-        <v>4000000</v>
-      </c>
-      <c r="G21" s="7">
-        <f>$J$6 *$O$8 / $L$6</f>
-        <v>64000</v>
-      </c>
-    </row>
-    <row r="22" spans="5:18" x14ac:dyDescent="0.3">
-      <c r="E22" s="8" t="s">
-        <v>442</v>
-      </c>
-      <c r="F22" s="8">
-        <f>$J$6 *$O$9 / $K$6</f>
-        <v>2000000</v>
-      </c>
-      <c r="G22" s="8">
-        <f>$J$6 *$O$9 / $L$6</f>
-        <v>32000</v>
-      </c>
-    </row>
-    <row r="23" spans="5:18" x14ac:dyDescent="0.3">
-      <c r="E23" s="7" t="s">
-        <v>443</v>
-      </c>
-      <c r="F23" s="7">
-        <f>$J$6 *$O$10 / $K$6</f>
-        <v>1000000</v>
-      </c>
-      <c r="G23" s="7">
-        <f>$J$6 *$O$10 / $L$6</f>
-        <v>16000</v>
-      </c>
-      <c r="R23" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="24" spans="5:18" x14ac:dyDescent="0.3">
-      <c r="E24" s="8" t="s">
-        <v>444</v>
-      </c>
-      <c r="F24" s="8">
-        <f>$J$6 *$O$11 / $K$6</f>
-        <v>500000</v>
-      </c>
-      <c r="G24" s="8">
-        <f>$J$6 *$O$11 / $L$6</f>
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="25" spans="5:18" x14ac:dyDescent="0.3">
-      <c r="E25" s="7" t="s">
-        <v>445</v>
-      </c>
-      <c r="F25" s="7">
-        <f>$J$6 *$O$12 / $K$6</f>
-        <v>250000</v>
-      </c>
-      <c r="G25" s="7">
-        <f>$J$6 *$O$12 / $L$6</f>
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="26" spans="5:18" x14ac:dyDescent="0.3">
-      <c r="E26" s="8" t="s">
-        <v>446</v>
-      </c>
-      <c r="F26" s="8">
-        <f>$J$6 *$O$13 / $K$6</f>
-        <v>125000</v>
-      </c>
-      <c r="G26" s="8">
-        <f>$J$6 *$O$13 / $L$6</f>
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="27" spans="5:18" x14ac:dyDescent="0.3">
-      <c r="E27" s="7" t="s">
-        <v>447</v>
-      </c>
-      <c r="F27" s="7">
-        <f>$J$6 / $O$14 / $K$6</f>
-        <v>62500</v>
-      </c>
-      <c r="G27" s="7">
-        <f>$J$6 / $O$14 / $L$6</f>
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="28" spans="5:18" x14ac:dyDescent="0.3">
-      <c r="E28" s="11" t="s">
-        <v>448</v>
-      </c>
-      <c r="F28" s="11">
-        <f>$J$6 / $O$15 / $K$6</f>
-        <v>31250</v>
-      </c>
-      <c r="G28" s="11">
-        <f>$J$6 / $O$15 / $L$6</f>
-        <v>500</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Update GenCode in FMKIO not properly...
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_designHRTIM\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84DB073-DCE4-41FB-B482-1AF0847BB781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493A8716-75C1-4D04-AF8F-FDC24DB2271E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="470">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="471">
   <si>
     <t>Colonne1</t>
   </si>
@@ -1448,13 +1448,16 @@
     <t>Timer Type</t>
   </si>
   <si>
-    <t>Tim</t>
-  </si>
-  <si>
     <t>HrTim</t>
   </si>
   <si>
     <t>TIMER_A</t>
+  </si>
+  <si>
+    <t>BscTim</t>
+  </si>
+  <si>
+    <t>AdvTim</t>
   </si>
 </sst>
 </file>
@@ -7057,7 +7060,7 @@
         <v>46</v>
       </c>
       <c r="U7" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="W7" t="s">
         <v>12</v>
@@ -7125,7 +7128,7 @@
         <v>92</v>
       </c>
       <c r="U8" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="W8" t="s">
         <v>12</v>
@@ -7193,7 +7196,7 @@
         <v>46</v>
       </c>
       <c r="U9" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="AA9" t="s">
         <v>12</v>
@@ -7252,7 +7255,7 @@
         <v>50</v>
       </c>
       <c r="U10" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="AA10" t="s">
         <v>12</v>
@@ -7296,7 +7299,7 @@
         <v>45</v>
       </c>
       <c r="U11" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="AA11" t="s">
         <v>12</v>
@@ -7328,7 +7331,7 @@
         <v>46</v>
       </c>
       <c r="U12" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="AA12" t="s">
         <v>12</v>
@@ -7360,7 +7363,7 @@
         <v>92</v>
       </c>
       <c r="U13" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="AA13" t="s">
         <v>11</v>
@@ -7392,7 +7395,7 @@
         <v>50</v>
       </c>
       <c r="U14" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="AA14" t="s">
         <v>11</v>
@@ -7418,7 +7421,7 @@
         <v>45</v>
       </c>
       <c r="U15" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="AA15" t="s">
         <v>11</v>
@@ -7444,7 +7447,7 @@
         <v>46</v>
       </c>
       <c r="U16" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="AA16" t="s">
         <v>14</v>
@@ -7464,13 +7467,13 @@
         <v>433</v>
       </c>
       <c r="S17" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="T17" t="s">
         <v>45</v>
       </c>
       <c r="U17" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="18" spans="1:53" x14ac:dyDescent="0.3">
@@ -7490,7 +7493,7 @@
         <v>50</v>
       </c>
       <c r="U18" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="24" spans="1:53" x14ac:dyDescent="0.3">
@@ -7830,7 +7833,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 K7:K10 Q7:Q14 F7:F11 B7:B14 X7:X8 AB8:AB16" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
       <formula1>$AW$30:$AW$45</formula1>
     </dataValidation>
@@ -7840,8 +7843,11 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7:H11" xr:uid="{FFFA1AF2-B35F-4BAA-AEF6-4A6121806F8D}">
       <formula1>$BA$30:$BA$47</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U7:U20" xr:uid="{843CAB93-5FB8-4584-AA77-D87D9BF50E6D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U19:U20" xr:uid="{843CAB93-5FB8-4584-AA77-D87D9BF50E6D}">
       <formula1>"HrTim,Tim"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U7:U18" xr:uid="{2E700A6E-F322-4D4F-87DE-D704594A5EA0}">
+      <formula1>"HrTim,BscTim,AdvTim"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Code Generation Done for Hrt/Io build OK, pulse not working
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_designHRTIM\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493A8716-75C1-4D04-AF8F-FDC24DB2271E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18C74771-62B7-43BF-98A8-66B4AF3D18B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1043" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="482">
   <si>
     <t>Colonne1</t>
   </si>
@@ -1343,27 +1343,18 @@
     <t>GPIO_AF4_TIM8</t>
   </si>
   <si>
-    <t>GPIO_AF6_TIM20</t>
-  </si>
-  <si>
     <t>GPIO_AF2_TIM4</t>
   </si>
   <si>
     <t>TIM8_UP_IRQHandler</t>
   </si>
   <si>
-    <t>EXTI2_IRQN</t>
-  </si>
-  <si>
     <t>EXTI9_5_IRQN</t>
   </si>
   <si>
     <t>JTAG User -&gt; PA14/PA13, PA15, PC1, PC0</t>
   </si>
   <si>
-    <t>GPIO_AF6_TIM1</t>
-  </si>
-  <si>
     <t>;</t>
   </si>
   <si>
@@ -1458,6 +1449,48 @@
   </si>
   <si>
     <t>AdvTim</t>
+  </si>
+  <si>
+    <t>GPIO_AF13_HRTIM1</t>
+  </si>
+  <si>
+    <t>TIMER_B</t>
+  </si>
+  <si>
+    <t>TIMER_C</t>
+  </si>
+  <si>
+    <t>TIMER_D</t>
+  </si>
+  <si>
+    <t>TIMER_E</t>
+  </si>
+  <si>
+    <t>TIMER_F</t>
+  </si>
+  <si>
+    <t>GPIO_AF3_HRTIM1</t>
+  </si>
+  <si>
+    <t>GPIO_AF3_TIM20</t>
+  </si>
+  <si>
+    <t>GPIO_AF1_TIM5</t>
+  </si>
+  <si>
+    <t>GPIO_AF1_TIM16</t>
+  </si>
+  <si>
+    <t>GPIO_AF1_TIM17</t>
+  </si>
+  <si>
+    <t>GPIO_AF1_TIM15</t>
+  </si>
+  <si>
+    <t>EXTI3_IRQN</t>
+  </si>
+  <si>
+    <t>EXTI4_IRQN</t>
   </si>
 </sst>
 </file>
@@ -1526,7 +1559,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1574,11 +1607,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1595,6 +1654,13 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4129,8 +4195,8 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}" name="FMKIO_InputDig" displayName="FMKIO_InputDig" ref="A6:B14" totalsRowShown="0">
-  <autoFilter ref="A6:B14" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}" name="FMKIO_InputDig" displayName="FMKIO_InputDig" ref="B6:C13" totalsRowShown="0">
+  <autoFilter ref="B6:C13" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{6C4BEFED-5E85-401A-AA66-51A07D13FEBC}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{E08F986F-8D6D-4DEB-A18F-F4FB9A36C956}" name="Pin_name"/>
@@ -4140,8 +4206,8 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}" name="FMKIO_OutputDig" displayName="FMKIO_OutputDig" ref="AA7:AB16" totalsRowShown="0">
-  <autoFilter ref="AA7:AB16" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}" name="FMKIO_OutputDig" displayName="FMKIO_OutputDig" ref="AA7:AB18" totalsRowShown="0">
+  <autoFilter ref="AA7:AB18" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{395BD36A-0840-48CF-8D8D-56878E366FC5}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{34DF2CF3-8826-4F9E-A09D-280EE0FEFFBB}" name="Pin_name"/>
@@ -4165,8 +4231,8 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}" name="FMKIO_InputEvnt" displayName="FMKIO_InputEvnt" ref="W6:Y8" totalsRowShown="0">
-  <autoFilter ref="W6:Y8" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}" name="FMKIO_InputEvnt" displayName="FMKIO_InputEvnt" ref="W6:Y9" totalsRowShown="0">
+  <autoFilter ref="W6:Y9" xr:uid="{0918A5C3-EE53-4DBF-8C0C-2251FB41871E}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5C8A98A4-9028-4F61-A263-67D85D1BFF84}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{D3F2DFB4-9CF8-4086-ABAA-63BD13D3A4C5}" name="Pin_name"/>
@@ -4177,8 +4243,8 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{DE41CD30-BCBD-40FE-B5DD-848DAAA9C25B}" name="FMKIO_OutputPwm" displayName="FMKIO_OutputPwm" ref="P6:U18" totalsRowShown="0">
-  <autoFilter ref="P6:U18" xr:uid="{DE41CD30-BCBD-40FE-B5DD-848DAAA9C25B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{DE41CD30-BCBD-40FE-B5DD-848DAAA9C25B}" name="FMKIO_OutputPwm" displayName="FMKIO_OutputPwm" ref="P6:U19" totalsRowShown="0">
+  <autoFilter ref="P6:U19" xr:uid="{DE41CD30-BCBD-40FE-B5DD-848DAAA9C25B}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{F2B685DB-87AE-429A-9E70-076DA856F9A2}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{30126296-E33C-4D56-9110-2D49FE159CF1}" name="Pin_name"/>
@@ -4192,8 +4258,8 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}" name="FMKIO_InputAna" displayName="FMKIO_InputAna" ref="E6:H11" totalsRowShown="0">
-  <autoFilter ref="E6:H11" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}" name="FMKIO_InputAna" displayName="FMKIO_InputAna" ref="E6:H10" totalsRowShown="0">
+  <autoFilter ref="E6:H10" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{EDBDBF14-1FA4-44B8-A62D-BAA9F312652A}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{75AD9B1E-8F88-4CD9-86AB-C0D6BFDB44CD}" name="Pin_name"/>
@@ -4852,13 +4918,13 @@
   <sheetData>
     <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="R17" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="S17" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="T17" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
@@ -6690,18 +6756,18 @@
   <sheetData>
     <row r="3" spans="2:15" ht="93.6" x14ac:dyDescent="1.75">
       <c r="B3" s="6" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.3">
       <c r="J5" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="K5" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="L5" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.3">
@@ -6757,18 +6823,18 @@
     </row>
     <row r="20" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E20" s="9" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="21" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E21" s="7" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F21" s="7">
         <f>$J$6 *$O$8 / $K$6</f>
@@ -6781,7 +6847,7 @@
     </row>
     <row r="22" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E22" s="8" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="F22" s="8">
         <f>$J$6 *$O$9 / $K$6</f>
@@ -6794,7 +6860,7 @@
     </row>
     <row r="23" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E23" s="7" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="F23" s="7">
         <f>$J$6 *$O$10 / $K$6</f>
@@ -6810,7 +6876,7 @@
     </row>
     <row r="24" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E24" s="8" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="F24" s="8">
         <f>$J$6 *$O$11 / $K$6</f>
@@ -6823,7 +6889,7 @@
     </row>
     <row r="25" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E25" s="7" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="F25" s="7">
         <f>$J$6 *$O$12 / $K$6</f>
@@ -6836,7 +6902,7 @@
     </row>
     <row r="26" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E26" s="8" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="F26" s="8">
         <f>$J$6 *$O$13 / $K$6</f>
@@ -6849,7 +6915,7 @@
     </row>
     <row r="27" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E27" s="7" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="F27" s="7">
         <f>$J$6 / $O$14 / $K$6</f>
@@ -6862,7 +6928,7 @@
     </row>
     <row r="28" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E28" s="11" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="F28" s="11">
         <f>$J$6 / $O$15 / $K$6</f>
@@ -6898,6 +6964,7 @@
     <col min="12" max="12" width="21.109375" customWidth="1"/>
     <col min="13" max="13" width="17.5546875" customWidth="1"/>
     <col min="14" max="14" width="18.109375" customWidth="1"/>
+    <col min="15" max="15" width="28.5546875" customWidth="1"/>
     <col min="16" max="16" width="24.6640625" customWidth="1"/>
     <col min="18" max="18" width="18.5546875" customWidth="1"/>
     <col min="19" max="19" width="23.33203125" customWidth="1"/>
@@ -6916,10 +6983,10 @@
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -6946,10 +7013,10 @@
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>23</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>24</v>
       </c>
       <c r="E6" t="s">
@@ -6995,7 +7062,7 @@
         <v>44</v>
       </c>
       <c r="U6" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="W6" t="s">
         <v>23</v>
@@ -7011,10 +7078,10 @@
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>35</v>
       </c>
       <c r="E7" t="s">
@@ -7045,31 +7112,31 @@
         <v>92</v>
       </c>
       <c r="P7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="R7" t="s">
-        <v>438</v>
+        <v>477</v>
       </c>
       <c r="S7" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="T7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="U7" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="W7" t="s">
         <v>12</v>
       </c>
       <c r="X7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="Y7" t="s">
-        <v>435</v>
+        <v>480</v>
       </c>
       <c r="AA7" t="s">
         <v>23</v>
@@ -7079,10 +7146,10 @@
       </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>36</v>
       </c>
       <c r="E8" t="s">
@@ -7113,22 +7180,22 @@
         <v>50</v>
       </c>
       <c r="P8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="R8" t="s">
-        <v>438</v>
+        <v>478</v>
       </c>
       <c r="S8" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="T8" t="s">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="U8" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="W8" t="s">
         <v>12</v>
@@ -7137,21 +7204,21 @@
         <v>30</v>
       </c>
       <c r="Y8" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="AA8" t="s">
         <v>12</v>
       </c>
       <c r="AB8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>13</v>
       </c>
-      <c r="B9" t="s">
-        <v>38</v>
+      <c r="C9" t="s">
+        <v>39</v>
       </c>
       <c r="E9" t="s">
         <v>11</v>
@@ -7169,48 +7236,57 @@
         <v>12</v>
       </c>
       <c r="K9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="L9" t="s">
-        <v>283</v>
+        <v>432</v>
       </c>
       <c r="M9" t="s">
-        <v>5</v>
+        <v>252</v>
       </c>
       <c r="N9" t="s">
         <v>45</v>
       </c>
-      <c r="P9" t="s">
+      <c r="P9" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="Q9" t="s">
-        <v>27</v>
-      </c>
-      <c r="R9" t="s">
-        <v>432</v>
-      </c>
-      <c r="S9" t="s">
-        <v>256</v>
-      </c>
-      <c r="T9" t="s">
+      <c r="Q9" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="R9" s="18" t="s">
+        <v>476</v>
+      </c>
+      <c r="S9" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="T9" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="U9" t="s">
-        <v>470</v>
+      <c r="U9" s="18" t="s">
+        <v>466</v>
+      </c>
+      <c r="W9" t="s">
+        <v>13</v>
+      </c>
+      <c r="X9" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y9" s="18" t="s">
+        <v>481</v>
       </c>
       <c r="AA9" t="s">
         <v>12</v>
       </c>
       <c r="AB9" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" t="s">
-        <v>39</v>
+      <c r="C10" t="s">
+        <v>40</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
@@ -7228,272 +7304,286 @@
         <v>12</v>
       </c>
       <c r="K10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="L10" t="s">
-        <v>283</v>
+        <v>432</v>
       </c>
       <c r="M10" t="s">
-        <v>5</v>
+        <v>252</v>
       </c>
       <c r="N10" t="s">
         <v>46</v>
       </c>
       <c r="P10" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>41</v>
+      </c>
+      <c r="R10" t="s">
+        <v>479</v>
+      </c>
+      <c r="S10" t="s">
+        <v>6</v>
+      </c>
+      <c r="T10" t="s">
+        <v>46</v>
+      </c>
+      <c r="U10" t="s">
+        <v>466</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
         <v>13</v>
       </c>
-      <c r="Q10" t="s">
-        <v>28</v>
-      </c>
-      <c r="R10" t="s">
-        <v>430</v>
-      </c>
-      <c r="S10" t="s">
-        <v>4</v>
-      </c>
-      <c r="T10" t="s">
-        <v>50</v>
-      </c>
-      <c r="U10" t="s">
-        <v>469</v>
-      </c>
-      <c r="AA10" t="s">
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="P11" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q11" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="R11" s="18" t="s">
+        <v>431</v>
+      </c>
+      <c r="S11" s="18" t="s">
+        <v>255</v>
+      </c>
+      <c r="T11" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="U11" s="18" t="s">
+        <v>467</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="P12" t="s">
         <v>12</v>
       </c>
-      <c r="AB10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" t="s">
-        <v>41</v>
-      </c>
-      <c r="G11" t="s">
-        <v>261</v>
-      </c>
-      <c r="H11" t="s">
-        <v>109</v>
-      </c>
-      <c r="P11" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>31</v>
-      </c>
-      <c r="R11" t="s">
-        <v>431</v>
-      </c>
-      <c r="S11" t="s">
-        <v>255</v>
-      </c>
-      <c r="T11" t="s">
+      <c r="Q12" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" t="s">
+        <v>475</v>
+      </c>
+      <c r="S12" t="s">
+        <v>256</v>
+      </c>
+      <c r="T12" t="s">
         <v>45</v>
       </c>
-      <c r="U11" t="s">
-        <v>470</v>
-      </c>
-      <c r="AA11" t="s">
-        <v>12</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>41</v>
-      </c>
-      <c r="P12" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>32</v>
-      </c>
-      <c r="R12" t="s">
-        <v>431</v>
-      </c>
-      <c r="S12" t="s">
-        <v>255</v>
-      </c>
-      <c r="T12" t="s">
-        <v>46</v>
-      </c>
       <c r="U12" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="AA12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AB12" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
         <v>11</v>
       </c>
-      <c r="B13" t="s">
-        <v>25</v>
+      <c r="C13" t="s">
+        <v>26</v>
       </c>
       <c r="P13" t="s">
         <v>13</v>
       </c>
       <c r="Q13" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="R13" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="S13" t="s">
-        <v>256</v>
+        <v>4</v>
       </c>
       <c r="T13" t="s">
         <v>92</v>
       </c>
       <c r="U13" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="AA13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AB13" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="P14" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B14" t="s">
+      <c r="Q14" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="R14" s="12" t="s">
+        <v>468</v>
+      </c>
+      <c r="S14" s="12" t="s">
+        <v>465</v>
+      </c>
+      <c r="T14" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="U14" s="13" t="s">
+        <v>464</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="P15" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q15" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="R15" s="15" t="s">
+        <v>468</v>
+      </c>
+      <c r="S15" s="15" t="s">
+        <v>469</v>
+      </c>
+      <c r="T15" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="U15" s="16" t="s">
+        <v>464</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="P16" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q16" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="R16" s="12" t="s">
+        <v>468</v>
+      </c>
+      <c r="S16" s="12" t="s">
+        <v>470</v>
+      </c>
+      <c r="T16" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="U16" s="13" t="s">
+        <v>464</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:53" x14ac:dyDescent="0.3">
+      <c r="P17" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q17" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="R17" s="15" t="s">
+        <v>468</v>
+      </c>
+      <c r="S17" s="15" t="s">
+        <v>471</v>
+      </c>
+      <c r="T17" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="U17" s="16" t="s">
+        <v>464</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>15</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:53" x14ac:dyDescent="0.3">
+      <c r="P18" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q18" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="R18" s="12" t="s">
+        <v>468</v>
+      </c>
+      <c r="S18" s="12" t="s">
+        <v>473</v>
+      </c>
+      <c r="T18" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="U18" s="13" t="s">
+        <v>464</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>15</v>
+      </c>
+      <c r="AB18" t="s">
         <v>26</v>
       </c>
-      <c r="P14" t="s">
+    </row>
+    <row r="19" spans="1:53" x14ac:dyDescent="0.3">
+      <c r="P19" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="Q14" t="s">
-        <v>34</v>
-      </c>
-      <c r="R14" t="s">
-        <v>431</v>
-      </c>
-      <c r="S14" t="s">
-        <v>255</v>
-      </c>
-      <c r="T14" t="s">
-        <v>50</v>
-      </c>
-      <c r="U14" t="s">
-        <v>470</v>
-      </c>
-      <c r="AA14" t="s">
-        <v>11</v>
-      </c>
-      <c r="AB14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="P15" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>31</v>
-      </c>
-      <c r="R15" t="s">
-        <v>433</v>
-      </c>
-      <c r="S15" t="s">
-        <v>252</v>
-      </c>
-      <c r="T15" t="s">
+      <c r="Q19" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="R19" s="15" t="s">
+        <v>474</v>
+      </c>
+      <c r="S19" s="15" t="s">
+        <v>472</v>
+      </c>
+      <c r="T19" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="U15" t="s">
-        <v>469</v>
-      </c>
-      <c r="AA15" t="s">
-        <v>11</v>
-      </c>
-      <c r="AB15" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="P16" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>32</v>
-      </c>
-      <c r="R16" t="s">
-        <v>433</v>
-      </c>
-      <c r="S16" t="s">
-        <v>252</v>
-      </c>
-      <c r="T16" t="s">
-        <v>46</v>
-      </c>
-      <c r="U16" t="s">
-        <v>469</v>
-      </c>
-      <c r="AA16" t="s">
-        <v>14</v>
-      </c>
-      <c r="AB16" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:53" x14ac:dyDescent="0.3">
-      <c r="P17" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>33</v>
-      </c>
-      <c r="R17" t="s">
-        <v>433</v>
-      </c>
-      <c r="S17" t="s">
-        <v>468</v>
-      </c>
-      <c r="T17" t="s">
-        <v>45</v>
-      </c>
-      <c r="U17" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="18" spans="1:53" x14ac:dyDescent="0.3">
-      <c r="P18" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>34</v>
-      </c>
-      <c r="R18" t="s">
-        <v>433</v>
-      </c>
-      <c r="S18" t="s">
-        <v>252</v>
-      </c>
-      <c r="T18" t="s">
-        <v>50</v>
-      </c>
-      <c r="U18" t="s">
-        <v>469</v>
+      <c r="U19" s="16" t="s">
+        <v>464</v>
       </c>
     </row>
     <row r="24" spans="1:53" x14ac:dyDescent="0.3">
@@ -7834,19 +7924,19 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 K7:K10 Q7:Q14 F7:F11 B7:B14 X7:X8 AB8:AB16" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 K7:K10 F7:F10 Q14:Q19 Q7 C7:C13 X7:X9 AB8:AB14 AB16:AB17" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
       <formula1>$AW$30:$AW$45</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N7:N10 T7:T14" xr:uid="{727A5344-B28A-4866-9EC1-7C96029AF8B6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N7:N10 T14:T19 T7" xr:uid="{727A5344-B28A-4866-9EC1-7C96029AF8B6}">
       <formula1>$AY$31:$AY$34</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7:H11" xr:uid="{FFFA1AF2-B35F-4BAA-AEF6-4A6121806F8D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7:H10" xr:uid="{FFFA1AF2-B35F-4BAA-AEF6-4A6121806F8D}">
       <formula1>$BA$30:$BA$47</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U19:U20" xr:uid="{843CAB93-5FB8-4584-AA77-D87D9BF50E6D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U21:U22" xr:uid="{843CAB93-5FB8-4584-AA77-D87D9BF50E6D}">
       <formula1>"HrTim,Tim"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U7:U18" xr:uid="{2E700A6E-F322-4D4F-87DE-D704594A5EA0}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U7 U12:U19" xr:uid="{2E700A6E-F322-4D4F-87DE-D704594A5EA0}">
       <formula1>"HrTim,BscTim,AdvTim"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7868,24 +7958,18 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{AA00DA78-9682-47F8-B701-D35809CE3FB0}">
           <x14:formula1>
             <xm:f>General_Info!$P$34:$P$39</xm:f>
           </x14:formula1>
-          <xm:sqref>P7:P14 J7:J10 E7:E11 A7:A14 W7:W8 AA8:AA16</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1C3D18C3-7241-4088-8034-07AAE0EB53A9}">
-          <x14:formula1>
-            <xm:f>General_Info!$K$19:$K$30</xm:f>
-          </x14:formula1>
-          <xm:sqref>S7:S14</xm:sqref>
+          <xm:sqref>J7:J10 E7:E10 P14:P19 P7 B7:B13 W7:W9 AA8:AA14 AA16:AA17</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C428027-B16D-4B04-9CB2-8290577ED0FB}">
           <x14:formula1>
             <xm:f>General_Info!$V$41:$V$45</xm:f>
           </x14:formula1>
-          <xm:sqref>G6:G11</xm:sqref>
+          <xm:sqref>G6:G10</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7928,7 +8012,7 @@
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>7</v>
+        <v>253</v>
       </c>
       <c r="C5" t="s">
         <v>45</v>
@@ -7942,7 +8026,7 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>8</v>
+        <v>254</v>
       </c>
       <c r="C6" t="s">
         <v>45</v>
@@ -8012,7 +8096,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="G14" t="s">
         <v>255</v>
@@ -8067,42 +8151,42 @@
     </row>
     <row r="6" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y6" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
     </row>
     <row r="7" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y7" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="8" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y8" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="9" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y9" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="10" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y10" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
     </row>
     <row r="11" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y11" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
     </row>
     <row r="12" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y12" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
     </row>
     <row r="13" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y13" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Validation commencer pour les PWM, ok pour toutes les sorties HighRes
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_designHRTIM\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18C74771-62B7-43BF-98A8-66B4AF3D18B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D55C8572-CACB-44FE-A84B-62E74AFE9A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="481">
   <si>
     <t>Colonne1</t>
   </si>
@@ -1422,9 +1422,6 @@
   </si>
   <si>
     <t>HRTIM1_Master_IRQHandler</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> HRTIM1_TIME_IRQHandler</t>
   </si>
   <si>
     <t>Hrtimer name</t>
@@ -1637,7 +1634,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1654,13 +1651,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4374,8 +4368,8 @@
 </file>
 
 <file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{953E7E02-522E-4F1F-B136-4D0BF069F045}" name="FMKHRT_IrqHandler" displayName="FMKHRT_IrqHandler" ref="Y5:Y13" totalsRowShown="0">
-  <autoFilter ref="Y5:Y13" xr:uid="{953E7E02-522E-4F1F-B136-4D0BF069F045}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{953E7E02-522E-4F1F-B136-4D0BF069F045}" name="FMKHRT_IrqHandler" displayName="FMKHRT_IrqHandler" ref="Y5:Y12" totalsRowShown="0">
+  <autoFilter ref="Y5:Y12" xr:uid="{953E7E02-522E-4F1F-B136-4D0BF069F045}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{4F3F9E81-1A81-491D-8B79-C106AA82CA37}" name="Colonne1"/>
   </tableColumns>
@@ -4918,13 +4912,13 @@
   <sheetData>
     <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="R17" t="s">
+        <v>459</v>
+      </c>
+      <c r="S17" t="s">
         <v>460</v>
       </c>
-      <c r="S17" t="s">
+      <c r="T17" t="s">
         <v>461</v>
-      </c>
-      <c r="T17" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
@@ -5187,7 +5181,7 @@
         <v>168</v>
       </c>
       <c r="N24" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="O24" t="s">
         <v>294</v>
@@ -5219,7 +5213,7 @@
         <v>169</v>
       </c>
       <c r="N25" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="O25" t="s">
         <v>295</v>
@@ -5289,7 +5283,7 @@
         <v>144</v>
       </c>
       <c r="N27" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="O27" t="s">
         <v>295</v>
@@ -5327,7 +5321,7 @@
         <v>145</v>
       </c>
       <c r="N28" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="O28" t="s">
         <v>295</v>
@@ -5365,7 +5359,7 @@
         <v>146</v>
       </c>
       <c r="N29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="O29" t="s">
         <v>295</v>
@@ -7062,7 +7056,7 @@
         <v>44</v>
       </c>
       <c r="U6" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="W6" t="s">
         <v>23</v>
@@ -7118,7 +7112,7 @@
         <v>29</v>
       </c>
       <c r="R7" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="S7" t="s">
         <v>7</v>
@@ -7127,7 +7121,7 @@
         <v>45</v>
       </c>
       <c r="U7" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="W7" t="s">
         <v>12</v>
@@ -7136,7 +7130,7 @@
         <v>28</v>
       </c>
       <c r="Y7" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="AA7" t="s">
         <v>23</v>
@@ -7186,7 +7180,7 @@
         <v>34</v>
       </c>
       <c r="R8" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="S8" t="s">
         <v>8</v>
@@ -7195,7 +7189,7 @@
         <v>45</v>
       </c>
       <c r="U8" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="W8" t="s">
         <v>12</v>
@@ -7247,23 +7241,23 @@
       <c r="N9" t="s">
         <v>45</v>
       </c>
-      <c r="P9" s="18" t="s">
+      <c r="P9" t="s">
         <v>13</v>
       </c>
-      <c r="Q9" s="18" t="s">
+      <c r="Q9" t="s">
         <v>38</v>
       </c>
-      <c r="R9" s="18" t="s">
-        <v>476</v>
-      </c>
-      <c r="S9" s="18" t="s">
+      <c r="R9" t="s">
+        <v>475</v>
+      </c>
+      <c r="S9" t="s">
         <v>257</v>
       </c>
-      <c r="T9" s="18" t="s">
+      <c r="T9" t="s">
         <v>46</v>
       </c>
-      <c r="U9" s="18" t="s">
-        <v>466</v>
+      <c r="U9" t="s">
+        <v>465</v>
       </c>
       <c r="W9" t="s">
         <v>13</v>
@@ -7271,8 +7265,8 @@
       <c r="X9" t="s">
         <v>29</v>
       </c>
-      <c r="Y9" s="18" t="s">
-        <v>481</v>
+      <c r="Y9" t="s">
+        <v>480</v>
       </c>
       <c r="AA9" t="s">
         <v>12</v>
@@ -7322,7 +7316,7 @@
         <v>41</v>
       </c>
       <c r="R10" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="S10" t="s">
         <v>6</v>
@@ -7331,7 +7325,7 @@
         <v>46</v>
       </c>
       <c r="U10" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="AA10" t="s">
         <v>11</v>
@@ -7347,23 +7341,23 @@
       <c r="C11" t="s">
         <v>41</v>
       </c>
-      <c r="P11" s="18" t="s">
+      <c r="P11" t="s">
         <v>13</v>
       </c>
-      <c r="Q11" s="18" t="s">
+      <c r="Q11" t="s">
         <v>32</v>
       </c>
-      <c r="R11" s="18" t="s">
+      <c r="R11" t="s">
         <v>431</v>
       </c>
-      <c r="S11" s="18" t="s">
+      <c r="S11" t="s">
         <v>255</v>
       </c>
-      <c r="T11" s="18" t="s">
+      <c r="T11" t="s">
         <v>46</v>
       </c>
-      <c r="U11" s="18" t="s">
-        <v>467</v>
+      <c r="U11" t="s">
+        <v>466</v>
       </c>
       <c r="AA11" t="s">
         <v>11</v>
@@ -7386,7 +7380,7 @@
         <v>27</v>
       </c>
       <c r="R12" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="S12" t="s">
         <v>256</v>
@@ -7395,7 +7389,7 @@
         <v>45</v>
       </c>
       <c r="U12" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="AA12" t="s">
         <v>11</v>
@@ -7427,7 +7421,7 @@
         <v>92</v>
       </c>
       <c r="U13" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="AA13" t="s">
         <v>12</v>
@@ -7437,23 +7431,23 @@
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="P14" s="14" t="s">
+      <c r="P14" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="Q14" s="12" t="s">
+      <c r="Q14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="R14" s="12" t="s">
-        <v>468</v>
-      </c>
-      <c r="S14" s="12" t="s">
-        <v>465</v>
-      </c>
-      <c r="T14" s="12" t="s">
+      <c r="R14" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="S14" s="7" t="s">
+        <v>464</v>
+      </c>
+      <c r="T14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="U14" s="13" t="s">
-        <v>464</v>
+      <c r="U14" s="12" t="s">
+        <v>463</v>
       </c>
       <c r="AA14" t="s">
         <v>13</v>
@@ -7463,23 +7457,23 @@
       </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="P15" s="17" t="s">
+      <c r="P15" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="Q15" s="15" t="s">
+      <c r="Q15" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="R15" s="15" t="s">
+      <c r="R15" s="8" t="s">
+        <v>467</v>
+      </c>
+      <c r="S15" s="8" t="s">
         <v>468</v>
       </c>
-      <c r="S15" s="15" t="s">
-        <v>469</v>
-      </c>
-      <c r="T15" s="15" t="s">
+      <c r="T15" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="U15" s="16" t="s">
-        <v>464</v>
+      <c r="U15" s="14" t="s">
+        <v>463</v>
       </c>
       <c r="AA15" t="s">
         <v>13</v>
@@ -7489,23 +7483,23 @@
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="P16" s="14" t="s">
+      <c r="P16" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="Q16" s="12" t="s">
+      <c r="Q16" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="R16" s="12" t="s">
-        <v>468</v>
-      </c>
-      <c r="S16" s="12" t="s">
-        <v>470</v>
-      </c>
-      <c r="T16" s="12" t="s">
+      <c r="R16" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="S16" s="7" t="s">
+        <v>469</v>
+      </c>
+      <c r="T16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="U16" s="13" t="s">
-        <v>464</v>
+      <c r="U16" s="12" t="s">
+        <v>463</v>
       </c>
       <c r="AA16" t="s">
         <v>13</v>
@@ -7515,23 +7509,23 @@
       </c>
     </row>
     <row r="17" spans="1:53" x14ac:dyDescent="0.3">
-      <c r="P17" s="17" t="s">
+      <c r="P17" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="Q17" s="15" t="s">
+      <c r="Q17" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="R17" s="15" t="s">
-        <v>468</v>
-      </c>
-      <c r="S17" s="15" t="s">
-        <v>471</v>
-      </c>
-      <c r="T17" s="15" t="s">
+      <c r="R17" s="8" t="s">
+        <v>467</v>
+      </c>
+      <c r="S17" s="8" t="s">
+        <v>470</v>
+      </c>
+      <c r="T17" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="U17" s="16" t="s">
-        <v>464</v>
+      <c r="U17" s="14" t="s">
+        <v>463</v>
       </c>
       <c r="AA17" t="s">
         <v>15</v>
@@ -7541,23 +7535,23 @@
       </c>
     </row>
     <row r="18" spans="1:53" x14ac:dyDescent="0.3">
-      <c r="P18" s="14" t="s">
+      <c r="P18" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="Q18" s="12" t="s">
+      <c r="Q18" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="R18" s="12" t="s">
-        <v>468</v>
-      </c>
-      <c r="S18" s="12" t="s">
-        <v>473</v>
-      </c>
-      <c r="T18" s="12" t="s">
+      <c r="R18" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="S18" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="T18" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="U18" s="13" t="s">
-        <v>464</v>
+      <c r="U18" s="12" t="s">
+        <v>463</v>
       </c>
       <c r="AA18" t="s">
         <v>15</v>
@@ -7567,23 +7561,23 @@
       </c>
     </row>
     <row r="19" spans="1:53" x14ac:dyDescent="0.3">
-      <c r="P19" s="17" t="s">
+      <c r="P19" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="Q19" s="15" t="s">
+      <c r="Q19" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="R19" s="15" t="s">
-        <v>474</v>
-      </c>
-      <c r="S19" s="15" t="s">
-        <v>472</v>
-      </c>
-      <c r="T19" s="15" t="s">
+      <c r="R19" s="8" t="s">
+        <v>473</v>
+      </c>
+      <c r="S19" s="8" t="s">
+        <v>471</v>
+      </c>
+      <c r="T19" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="U19" s="16" t="s">
-        <v>464</v>
+      <c r="U19" s="14" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="24" spans="1:53" x14ac:dyDescent="0.3">
@@ -8138,7 +8132,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BF150CB-3330-4180-96AC-4A3D28CDB7F6}">
-  <dimension ref="Y5:Y13"/>
+  <dimension ref="Y5:Y12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="25" max="25" width="27.21875" customWidth="1"/>
@@ -8182,11 +8176,6 @@
     <row r="12" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y12" t="s">
         <v>458</v>
-      </c>
-    </row>
-    <row r="13" spans="25:25" x14ac:dyDescent="0.3">
-      <c r="Y13" t="s">
-        <v>459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
testing adc not working
</commit_message>
<xml_diff>
--- a/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
+++ b/Doc/ConfigPrj/ExcelCfg/STM32G474RE/STM32G474RE_HwCfg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Software\STM32\f_designHRTIM\Doc\ConfigPrj\ExcelCfg\STM32G474RE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D55C8572-CACB-44FE-A84B-62E74AFE9A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390137E0-CC7D-4D1C-B8E2-19DC12920407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{2AF09063-600F-437A-B138-F66136E922A5}"/>
   </bookViews>
   <sheets>
     <sheet name="General_Info" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1049" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1057" uniqueCount="480">
   <si>
     <t>Colonne1</t>
   </si>
@@ -894,9 +894,6 @@
   </si>
   <si>
     <t>Reference to AlternateFunction Datasheet</t>
-  </si>
-  <si>
-    <t>GPIO_AF2_TIM3</t>
   </si>
   <si>
     <t>GPIO_AF9_FDCAN1</t>
@@ -4189,8 +4186,8 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}" name="FMKIO_InputDig" displayName="FMKIO_InputDig" ref="B6:C13" totalsRowShown="0">
-  <autoFilter ref="B6:C13" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}" name="FMKIO_InputDig" displayName="FMKIO_InputDig" ref="A6:B15" totalsRowShown="0">
+  <autoFilter ref="A6:B15" xr:uid="{9F4B7C8E-8730-4908-B1BE-2954AF9427C0}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{6C4BEFED-5E85-401A-AA66-51A07D13FEBC}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{E08F986F-8D6D-4DEB-A18F-F4FB9A36C956}" name="Pin_name"/>
@@ -4200,8 +4197,8 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}" name="FMKIO_OutputDig" displayName="FMKIO_OutputDig" ref="AA7:AB18" totalsRowShown="0">
-  <autoFilter ref="AA7:AB18" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}" name="FMKIO_OutputDig" displayName="FMKIO_OutputDig" ref="AA7:AB17" totalsRowShown="0">
+  <autoFilter ref="AA7:AB17" xr:uid="{098A48DC-88A9-4122-ADE1-86E0F3796141}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{395BD36A-0840-48CF-8D8D-56878E366FC5}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{34DF2CF3-8826-4F9E-A09D-280EE0FEFFBB}" name="Pin_name"/>
@@ -4211,8 +4208,8 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{27D0C574-E325-48F5-AA31-7FBAF1E09007}" name="FMKIO_InputFreq" displayName="FMKIO_InputFreq" ref="J6:N10" totalsRowShown="0">
-  <autoFilter ref="J6:N10" xr:uid="{27D0C574-E325-48F5-AA31-7FBAF1E09007}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{27D0C574-E325-48F5-AA31-7FBAF1E09007}" name="FMKIO_InputFreq" displayName="FMKIO_InputFreq" ref="J6:N8" totalsRowShown="0">
+  <autoFilter ref="J6:N8" xr:uid="{27D0C574-E325-48F5-AA31-7FBAF1E09007}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{F1DD33F7-0EF3-4BDF-839A-2E3FA15D0FD7}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{1EC5875F-046C-4961-B678-CB3386C5E012}" name="Pin_name"/>
@@ -4252,8 +4249,8 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}" name="FMKIO_InputAna" displayName="FMKIO_InputAna" ref="E6:H10" totalsRowShown="0">
-  <autoFilter ref="E6:H10" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}" name="FMKIO_InputAna" displayName="FMKIO_InputAna" ref="E6:H12" totalsRowShown="0">
+  <autoFilter ref="E6:H12" xr:uid="{B6D8F853-4E95-4D0E-932E-0F3ECC221901}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{EDBDBF14-1FA4-44B8-A62D-BAA9F312652A}" name="GPIO_name"/>
     <tableColumn id="2" xr3:uid="{75AD9B1E-8F88-4CD9-86AB-C0D6BFDB44CD}" name="Pin_name"/>
@@ -4426,8 +4423,8 @@
 </file>
 
 <file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}" name="FMKMAC_Cfg" displayName="FMKMAC_Cfg" ref="B2:E12" totalsRowShown="0">
-  <autoFilter ref="B2:E12" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}" name="FMKMAC_Cfg" displayName="FMKMAC_Cfg" ref="B2:E14" totalsRowShown="0">
+  <autoFilter ref="B2:E14" xr:uid="{333A4E38-7E7A-4098-B282-4F58DD308AC2}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{9B6EDCAA-F526-412C-A8EC-AC6897A0EB04}" name="RqstDmaType"/>
     <tableColumn id="2" xr3:uid="{ED583461-6D2B-456F-A394-15F76B273D8C}" name="DMA "/>
@@ -4912,13 +4909,13 @@
   <sheetData>
     <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="R17" t="s">
+        <v>458</v>
+      </c>
+      <c r="S17" t="s">
         <v>459</v>
       </c>
-      <c r="S17" t="s">
+      <c r="T17" t="s">
         <v>460</v>
-      </c>
-      <c r="T17" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
@@ -4929,10 +4926,10 @@
         <v>21</v>
       </c>
       <c r="E18" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F18" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H18" t="s">
         <v>57</v>
@@ -4953,7 +4950,7 @@
         <v>270</v>
       </c>
       <c r="O18" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="R18" t="s">
         <v>250</v>
@@ -4973,10 +4970,10 @@
         <v>85</v>
       </c>
       <c r="E19" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F19" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H19" t="s">
         <v>59</v>
@@ -4997,7 +4994,7 @@
         <v>272</v>
       </c>
       <c r="O19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.3">
@@ -5005,10 +5002,10 @@
         <v>230</v>
       </c>
       <c r="E20" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F20" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H20" t="s">
         <v>124</v>
@@ -5029,7 +5026,7 @@
         <v>272</v>
       </c>
       <c r="O20" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="AB20" t="s">
         <v>22</v>
@@ -5046,10 +5043,10 @@
         <v>233</v>
       </c>
       <c r="E21" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F21" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H21" t="s">
         <v>125</v>
@@ -5070,10 +5067,10 @@
         <v>272</v>
       </c>
       <c r="O21" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="AB21" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="AC21">
         <v>8</v>
@@ -5087,10 +5084,10 @@
         <v>234</v>
       </c>
       <c r="E22" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F22" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H22" t="s">
         <v>126</v>
@@ -5111,10 +5108,10 @@
         <v>272</v>
       </c>
       <c r="O22" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="AB22" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AC22">
         <v>8</v>
@@ -5128,10 +5125,10 @@
         <v>235</v>
       </c>
       <c r="E23" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F23" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H23" t="s">
         <v>60</v>
@@ -5152,7 +5149,7 @@
         <v>272</v>
       </c>
       <c r="O23" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.3">
@@ -5160,10 +5157,10 @@
         <v>236</v>
       </c>
       <c r="E24" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F24" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H24" t="s">
         <v>61</v>
@@ -5184,7 +5181,7 @@
         <v>273</v>
       </c>
       <c r="O24" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="25" spans="1:30" x14ac:dyDescent="0.3">
@@ -5192,10 +5189,10 @@
         <v>84</v>
       </c>
       <c r="E25" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F25" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H25" t="s">
         <v>127</v>
@@ -5216,7 +5213,7 @@
         <v>273</v>
       </c>
       <c r="O25" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="26" spans="1:30" x14ac:dyDescent="0.3">
@@ -5224,10 +5221,10 @@
         <v>260</v>
       </c>
       <c r="E26" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F26" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H26" t="s">
         <v>128</v>
@@ -5248,7 +5245,7 @@
         <v>272</v>
       </c>
       <c r="O26" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="27" spans="1:30" x14ac:dyDescent="0.3">
@@ -5262,10 +5259,10 @@
         <v>83</v>
       </c>
       <c r="E27" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F27" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H27" t="s">
         <v>129</v>
@@ -5286,7 +5283,7 @@
         <v>272</v>
       </c>
       <c r="O27" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.3">
@@ -5300,10 +5297,10 @@
         <v>231</v>
       </c>
       <c r="E28" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F28" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H28" t="s">
         <v>130</v>
@@ -5324,7 +5321,7 @@
         <v>272</v>
       </c>
       <c r="O28" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="29" spans="1:30" x14ac:dyDescent="0.3">
@@ -5338,10 +5335,10 @@
         <v>232</v>
       </c>
       <c r="E29" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F29" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H29" t="s">
         <v>131</v>
@@ -5362,7 +5359,7 @@
         <v>272</v>
       </c>
       <c r="O29" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.3">
@@ -5370,10 +5367,10 @@
         <v>82</v>
       </c>
       <c r="E30" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F30" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H30" t="s">
         <v>62</v>
@@ -5394,7 +5391,7 @@
         <v>272</v>
       </c>
       <c r="O30" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.3">
@@ -5402,10 +5399,10 @@
         <v>81</v>
       </c>
       <c r="E31" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F31" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H31" t="s">
         <v>132</v>
@@ -5419,10 +5416,10 @@
         <v>80</v>
       </c>
       <c r="E32" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F32" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H32" t="s">
         <v>133</v>
@@ -5436,10 +5433,10 @@
         <v>237</v>
       </c>
       <c r="E33" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F33" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H33" t="s">
         <v>134</v>
@@ -5459,10 +5456,10 @@
         <v>238</v>
       </c>
       <c r="E34" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F34" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H34" t="s">
         <v>135</v>
@@ -5482,10 +5479,10 @@
         <v>229</v>
       </c>
       <c r="E35" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F35" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H35" t="s">
         <v>136</v>
@@ -5505,10 +5502,10 @@
         <v>228</v>
       </c>
       <c r="E36" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F36" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H36" t="s">
         <v>137</v>
@@ -5534,10 +5531,10 @@
         <v>239</v>
       </c>
       <c r="E37" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F37" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H37" t="s">
         <v>138</v>
@@ -5563,10 +5560,10 @@
         <v>240</v>
       </c>
       <c r="E38" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F38" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H38" t="s">
         <v>139</v>
@@ -5586,10 +5583,10 @@
         <v>215</v>
       </c>
       <c r="E39" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F39" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H39" t="s">
         <v>140</v>
@@ -5609,10 +5606,10 @@
         <v>241</v>
       </c>
       <c r="E40" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F40" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H40" t="s">
         <v>141</v>
@@ -5647,10 +5644,10 @@
         <v>242</v>
       </c>
       <c r="E41" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F41" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H41" t="s">
         <v>142</v>
@@ -5679,10 +5676,10 @@
         <v>227</v>
       </c>
       <c r="E42" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F42" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H42" t="s">
         <v>143</v>
@@ -5711,10 +5708,10 @@
         <v>72</v>
       </c>
       <c r="E43" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F43" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H43" t="s">
         <v>144</v>
@@ -5743,10 +5740,10 @@
         <v>226</v>
       </c>
       <c r="E44" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F44" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H44" t="s">
         <v>145</v>
@@ -5772,10 +5769,10 @@
         <v>243</v>
       </c>
       <c r="E45" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F45" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H45" t="s">
         <v>146</v>
@@ -5801,10 +5798,10 @@
         <v>225</v>
       </c>
       <c r="E46" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F46" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H46" t="s">
         <v>63</v>
@@ -5821,10 +5818,10 @@
         <v>224</v>
       </c>
       <c r="E47" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F47" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H47" t="s">
         <v>147</v>
@@ -5841,10 +5838,10 @@
         <v>244</v>
       </c>
       <c r="E48" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F48" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H48" t="s">
         <v>64</v>
@@ -5861,10 +5858,10 @@
         <v>245</v>
       </c>
       <c r="E49" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F49" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H49" t="s">
         <v>148</v>
@@ -5881,10 +5878,10 @@
         <v>86</v>
       </c>
       <c r="E50" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F50" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H50" t="s">
         <v>149</v>
@@ -5898,10 +5895,10 @@
         <v>77</v>
       </c>
       <c r="E51" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F51" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H51" t="s">
         <v>150</v>
@@ -5915,10 +5912,10 @@
         <v>220</v>
       </c>
       <c r="E52" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F52" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H52" t="s">
         <v>151</v>
@@ -5927,7 +5924,7 @@
         <v>69</v>
       </c>
       <c r="AF52" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="53" spans="4:32" x14ac:dyDescent="0.3">
@@ -5935,10 +5932,10 @@
         <v>79</v>
       </c>
       <c r="E53" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F53" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H53" t="s">
         <v>152</v>
@@ -5947,7 +5944,7 @@
         <v>69</v>
       </c>
       <c r="AF53" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="54" spans="4:32" x14ac:dyDescent="0.3">
@@ -5955,10 +5952,10 @@
         <v>219</v>
       </c>
       <c r="E54" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F54" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H54" t="s">
         <v>65</v>
@@ -5967,7 +5964,7 @@
         <v>69</v>
       </c>
       <c r="AF54" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="55" spans="4:32" x14ac:dyDescent="0.3">
@@ -5975,10 +5972,10 @@
         <v>277</v>
       </c>
       <c r="E55" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F55" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H55" t="s">
         <v>66</v>
@@ -5987,7 +5984,7 @@
         <v>69</v>
       </c>
       <c r="AF55" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="56" spans="4:32" x14ac:dyDescent="0.3">
@@ -5995,10 +5992,10 @@
         <v>278</v>
       </c>
       <c r="E56" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F56" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H56" t="s">
         <v>67</v>
@@ -6007,7 +6004,7 @@
         <v>69</v>
       </c>
       <c r="AF56" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="57" spans="4:32" x14ac:dyDescent="0.3">
@@ -6015,10 +6012,10 @@
         <v>218</v>
       </c>
       <c r="E57" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F57" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H57" t="s">
         <v>68</v>
@@ -6027,7 +6024,7 @@
         <v>69</v>
       </c>
       <c r="AF57" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="58" spans="4:32" x14ac:dyDescent="0.3">
@@ -6035,10 +6032,10 @@
         <v>216</v>
       </c>
       <c r="E58" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F58" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H58" t="s">
         <v>153</v>
@@ -6047,7 +6044,7 @@
         <v>69</v>
       </c>
       <c r="AF58" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="59" spans="4:32" x14ac:dyDescent="0.3">
@@ -6055,10 +6052,10 @@
         <v>246</v>
       </c>
       <c r="E59" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F59" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H59" t="s">
         <v>154</v>
@@ -6067,7 +6064,7 @@
         <v>69</v>
       </c>
       <c r="AF59" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="60" spans="4:32" x14ac:dyDescent="0.3">
@@ -6075,10 +6072,10 @@
         <v>87</v>
       </c>
       <c r="E60" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F60" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H60" t="s">
         <v>155</v>
@@ -6087,7 +6084,7 @@
         <v>69</v>
       </c>
       <c r="AF60" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="61" spans="4:32" x14ac:dyDescent="0.3">
@@ -6095,10 +6092,10 @@
         <v>217</v>
       </c>
       <c r="E61" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F61" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H61" t="s">
         <v>156</v>
@@ -6107,7 +6104,7 @@
         <v>69</v>
       </c>
       <c r="AF61" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="62" spans="4:32" x14ac:dyDescent="0.3">
@@ -6115,10 +6112,10 @@
         <v>221</v>
       </c>
       <c r="E62" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F62" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H62" t="s">
         <v>157</v>
@@ -6127,7 +6124,7 @@
         <v>69</v>
       </c>
       <c r="AF62" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="63" spans="4:32" x14ac:dyDescent="0.3">
@@ -6135,10 +6132,10 @@
         <v>247</v>
       </c>
       <c r="E63" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F63" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H63" t="s">
         <v>158</v>
@@ -6152,10 +6149,10 @@
         <v>70</v>
       </c>
       <c r="E64" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F64" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H64" t="s">
         <v>159</v>
@@ -6169,10 +6166,10 @@
         <v>71</v>
       </c>
       <c r="E65" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F65" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H65" t="s">
         <v>160</v>
@@ -6186,10 +6183,10 @@
         <v>76</v>
       </c>
       <c r="E66" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F66" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H66" t="s">
         <v>161</v>
@@ -6203,10 +6200,10 @@
         <v>223</v>
       </c>
       <c r="E67" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F67" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H67" t="s">
         <v>162</v>
@@ -6220,10 +6217,10 @@
         <v>78</v>
       </c>
       <c r="E68" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F68" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H68" t="s">
         <v>163</v>
@@ -6237,10 +6234,10 @@
         <v>248</v>
       </c>
       <c r="E69" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F69" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H69" t="s">
         <v>164</v>
@@ -6254,10 +6251,10 @@
         <v>73</v>
       </c>
       <c r="E70" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F70" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H70" t="s">
         <v>165</v>
@@ -6271,10 +6268,10 @@
         <v>74</v>
       </c>
       <c r="E71" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F71" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H71" t="s">
         <v>166</v>
@@ -6288,10 +6285,10 @@
         <v>75</v>
       </c>
       <c r="E72" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F72" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H72" t="s">
         <v>167</v>
@@ -6305,10 +6302,10 @@
         <v>222</v>
       </c>
       <c r="E73" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F73" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H73" t="s">
         <v>168</v>
@@ -6322,10 +6319,10 @@
         <v>249</v>
       </c>
       <c r="E74" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F74" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H74" t="s">
         <v>169</v>
@@ -6339,10 +6336,10 @@
         <v>250</v>
       </c>
       <c r="E75" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F75" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="H75" t="s">
         <v>170</v>
@@ -6750,18 +6747,18 @@
   <sheetData>
     <row r="3" spans="2:15" ht="93.6" x14ac:dyDescent="1.75">
       <c r="B3" s="6" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.3">
       <c r="J5" t="s">
+        <v>448</v>
+      </c>
+      <c r="K5" t="s">
         <v>449</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>450</v>
-      </c>
-      <c r="L5" t="s">
-        <v>451</v>
       </c>
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.3">
@@ -6817,18 +6814,18 @@
     </row>
     <row r="20" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E20" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="G20" s="10" t="s">
         <v>446</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>448</v>
-      </c>
-      <c r="G20" s="10" t="s">
-        <v>447</v>
       </c>
     </row>
     <row r="21" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E21" s="7" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="F21" s="7">
         <f>$J$6 *$O$8 / $K$6</f>
@@ -6841,7 +6838,7 @@
     </row>
     <row r="22" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E22" s="8" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="F22" s="8">
         <f>$J$6 *$O$9 / $K$6</f>
@@ -6854,7 +6851,7 @@
     </row>
     <row r="23" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E23" s="7" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="F23" s="7">
         <f>$J$6 *$O$10 / $K$6</f>
@@ -6870,7 +6867,7 @@
     </row>
     <row r="24" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E24" s="8" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="F24" s="8">
         <f>$J$6 *$O$11 / $K$6</f>
@@ -6883,7 +6880,7 @@
     </row>
     <row r="25" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E25" s="7" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F25" s="7">
         <f>$J$6 *$O$12 / $K$6</f>
@@ -6896,7 +6893,7 @@
     </row>
     <row r="26" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E26" s="8" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="F26" s="8">
         <f>$J$6 *$O$13 / $K$6</f>
@@ -6909,7 +6906,7 @@
     </row>
     <row r="27" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E27" s="7" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F27" s="7">
         <f>$J$6 / $O$14 / $K$6</f>
@@ -6922,7 +6919,7 @@
     </row>
     <row r="28" spans="5:18" x14ac:dyDescent="0.3">
       <c r="E28" s="11" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F28" s="11">
         <f>$J$6 / $O$15 / $K$6</f>
@@ -6977,10 +6974,10 @@
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.3">
@@ -7007,10 +7004,10 @@
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
       <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
         <v>24</v>
       </c>
       <c r="E6" t="s">
@@ -7056,7 +7053,7 @@
         <v>44</v>
       </c>
       <c r="U6" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="W6" t="s">
         <v>23</v>
@@ -7072,38 +7069,38 @@
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
       <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" t="s">
         <v>35</v>
       </c>
       <c r="E7" t="s">
         <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>261</v>
+        <v>16</v>
       </c>
       <c r="H7" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="J7" t="s">
         <v>12</v>
       </c>
       <c r="K7" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="L7" t="s">
-        <v>283</v>
+        <v>431</v>
       </c>
       <c r="M7" t="s">
-        <v>5</v>
+        <v>252</v>
       </c>
       <c r="N7" t="s">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="P7" t="s">
         <v>12</v>
@@ -7112,7 +7109,7 @@
         <v>29</v>
       </c>
       <c r="R7" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="S7" t="s">
         <v>7</v>
@@ -7121,7 +7118,7 @@
         <v>45</v>
       </c>
       <c r="U7" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="W7" t="s">
         <v>12</v>
@@ -7130,7 +7127,7 @@
         <v>28</v>
       </c>
       <c r="Y7" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="AA7" t="s">
         <v>23</v>
@@ -7140,38 +7137,38 @@
       </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
       <c r="B8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" t="s">
         <v>36</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G8" t="s">
         <v>261</v>
       </c>
       <c r="H8" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="J8" t="s">
         <v>12</v>
       </c>
       <c r="K8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="L8" t="s">
-        <v>283</v>
+        <v>431</v>
       </c>
       <c r="M8" t="s">
-        <v>5</v>
+        <v>252</v>
       </c>
       <c r="N8" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="P8" t="s">
         <v>12</v>
@@ -7180,7 +7177,7 @@
         <v>34</v>
       </c>
       <c r="R8" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="S8" t="s">
         <v>8</v>
@@ -7189,7 +7186,7 @@
         <v>45</v>
       </c>
       <c r="U8" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="W8" t="s">
         <v>12</v>
@@ -7198,7 +7195,7 @@
         <v>30</v>
       </c>
       <c r="Y8" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="AA8" t="s">
         <v>12</v>
@@ -7208,38 +7205,23 @@
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
       <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" t="s">
         <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>261</v>
+        <v>16</v>
       </c>
       <c r="H9" t="s">
-        <v>97</v>
-      </c>
-      <c r="J9" t="s">
-        <v>12</v>
-      </c>
-      <c r="K9" t="s">
-        <v>31</v>
-      </c>
-      <c r="L9" t="s">
-        <v>432</v>
-      </c>
-      <c r="M9" t="s">
-        <v>252</v>
-      </c>
-      <c r="N9" t="s">
-        <v>45</v>
+        <v>106</v>
       </c>
       <c r="P9" t="s">
         <v>13</v>
@@ -7248,7 +7230,7 @@
         <v>38</v>
       </c>
       <c r="R9" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="S9" t="s">
         <v>257</v>
@@ -7257,7 +7239,7 @@
         <v>46</v>
       </c>
       <c r="U9" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="W9" t="s">
         <v>13</v>
@@ -7266,48 +7248,33 @@
         <v>29</v>
       </c>
       <c r="Y9" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="AA9" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s">
         <v>12</v>
       </c>
-      <c r="AB9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" t="s">
-        <v>11</v>
-      </c>
       <c r="F10" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>261</v>
+        <v>16</v>
       </c>
       <c r="H10" t="s">
-        <v>98</v>
-      </c>
-      <c r="J10" t="s">
-        <v>12</v>
-      </c>
-      <c r="K10" t="s">
-        <v>32</v>
-      </c>
-      <c r="L10" t="s">
-        <v>432</v>
-      </c>
-      <c r="M10" t="s">
-        <v>252</v>
-      </c>
-      <c r="N10" t="s">
-        <v>46</v>
+        <v>109</v>
       </c>
       <c r="P10" t="s">
         <v>12</v>
@@ -7316,7 +7283,7 @@
         <v>41</v>
       </c>
       <c r="R10" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="S10" t="s">
         <v>6</v>
@@ -7325,21 +7292,33 @@
         <v>46</v>
       </c>
       <c r="U10" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="AA10" t="s">
         <v>11</v>
       </c>
       <c r="AB10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
       <c r="B11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" t="s">
         <v>41</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
+        <v>30</v>
+      </c>
+      <c r="G11" t="s">
+        <v>261</v>
+      </c>
+      <c r="H11" t="s">
+        <v>107</v>
       </c>
       <c r="P11" t="s">
         <v>13</v>
@@ -7348,7 +7327,7 @@
         <v>32</v>
       </c>
       <c r="R11" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="S11" t="s">
         <v>255</v>
@@ -7357,21 +7336,33 @@
         <v>46</v>
       </c>
       <c r="U11" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="AA11" t="s">
         <v>11</v>
       </c>
       <c r="AB11" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
       <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" t="s">
         <v>11</v>
       </c>
-      <c r="C12" t="s">
-        <v>25</v>
+      <c r="F12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" t="s">
+        <v>261</v>
+      </c>
+      <c r="H12" t="s">
+        <v>97</v>
       </c>
       <c r="P12" t="s">
         <v>12</v>
@@ -7380,7 +7371,7 @@
         <v>27</v>
       </c>
       <c r="R12" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="S12" t="s">
         <v>256</v>
@@ -7389,21 +7380,21 @@
         <v>45</v>
       </c>
       <c r="U12" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="AA12" t="s">
+        <v>12</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="AB12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="P13" t="s">
         <v>13</v>
@@ -7412,7 +7403,7 @@
         <v>27</v>
       </c>
       <c r="R13" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="S13" t="s">
         <v>4</v>
@@ -7421,16 +7412,22 @@
         <v>92</v>
       </c>
       <c r="U13" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="AA13" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="AB13" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>35</v>
+      </c>
       <c r="P14" s="13" t="s">
         <v>11</v>
       </c>
@@ -7438,25 +7435,31 @@
         <v>33</v>
       </c>
       <c r="R14" s="7" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="S14" s="7" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="T14" s="7" t="s">
         <v>45</v>
       </c>
       <c r="U14" s="12" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="AA14" t="s">
         <v>13</v>
       </c>
       <c r="AB14" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>39</v>
+      </c>
       <c r="P15" s="15" t="s">
         <v>11</v>
       </c>
@@ -7464,22 +7467,22 @@
         <v>35</v>
       </c>
       <c r="R15" s="8" t="s">
+        <v>466</v>
+      </c>
+      <c r="S15" s="8" t="s">
         <v>467</v>
-      </c>
-      <c r="S15" s="8" t="s">
-        <v>468</v>
       </c>
       <c r="T15" s="8" t="s">
         <v>45</v>
       </c>
       <c r="U15" s="14" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="AA15" t="s">
         <v>13</v>
       </c>
       <c r="AB15" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.3">
@@ -7490,22 +7493,22 @@
         <v>38</v>
       </c>
       <c r="R16" s="7" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="S16" s="7" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="T16" s="7" t="s">
         <v>45</v>
       </c>
       <c r="U16" s="12" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="AA16" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="AB16" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:53" x14ac:dyDescent="0.3">
@@ -7516,22 +7519,22 @@
         <v>40</v>
       </c>
       <c r="R17" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="S17" s="8" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="T17" s="8" t="s">
         <v>45</v>
       </c>
       <c r="U17" s="14" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="AA17" t="s">
         <v>15</v>
       </c>
       <c r="AB17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:53" x14ac:dyDescent="0.3">
@@ -7542,22 +7545,16 @@
         <v>31</v>
       </c>
       <c r="R18" s="7" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="S18" s="7" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="T18" s="7" t="s">
         <v>45</v>
       </c>
       <c r="U18" s="12" t="s">
-        <v>463</v>
-      </c>
-      <c r="AA18" t="s">
-        <v>15</v>
-      </c>
-      <c r="AB18" t="s">
-        <v>26</v>
+        <v>462</v>
       </c>
     </row>
     <row r="19" spans="1:53" x14ac:dyDescent="0.3">
@@ -7568,41 +7565,41 @@
         <v>33</v>
       </c>
       <c r="R19" s="8" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="S19" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="T19" s="8" t="s">
         <v>45</v>
       </c>
       <c r="U19" s="14" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="24" spans="1:53" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="25" spans="1:53" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>284</v>
+      </c>
+      <c r="B25" t="s">
         <v>285</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>286</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>287</v>
-      </c>
-      <c r="D25" t="s">
-        <v>288</v>
       </c>
       <c r="E25" t="s">
         <v>42</v>
       </c>
       <c r="F25" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="26" spans="1:53" x14ac:dyDescent="0.3">
@@ -7619,10 +7616,10 @@
         <v>38</v>
       </c>
       <c r="E26" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F26" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="27" spans="1:53" x14ac:dyDescent="0.3">
@@ -7639,10 +7636,10 @@
         <v>41</v>
       </c>
       <c r="E27" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F27" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="28" spans="1:53" x14ac:dyDescent="0.3">
@@ -7659,18 +7656,18 @@
         <v>38</v>
       </c>
       <c r="E28" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F28" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="W28" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="29" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W29" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="AW29" t="s">
         <v>91</v>
@@ -7681,7 +7678,7 @@
     </row>
     <row r="30" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W30" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="AW30" t="s">
         <v>25</v>
@@ -7695,7 +7692,7 @@
     </row>
     <row r="31" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W31" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AW31" t="s">
         <v>26</v>
@@ -7709,7 +7706,7 @@
     </row>
     <row r="32" spans="1:53" x14ac:dyDescent="0.3">
       <c r="W32" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AW32" t="s">
         <v>27</v>
@@ -7723,10 +7720,10 @@
     </row>
     <row r="33" spans="1:53" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="W33" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AW33" t="s">
         <v>28</v>
@@ -7740,25 +7737,25 @@
     </row>
     <row r="34" spans="1:53" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>284</v>
+      </c>
+      <c r="B34" t="s">
         <v>285</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>286</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>287</v>
-      </c>
-      <c r="D34" t="s">
-        <v>288</v>
       </c>
       <c r="E34" t="s">
         <v>42</v>
       </c>
       <c r="F34" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="W34" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="AW34" t="s">
         <v>29</v>
@@ -7784,13 +7781,13 @@
         <v>27</v>
       </c>
       <c r="E35" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F35" t="s">
         <v>79</v>
       </c>
       <c r="W35" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AW35" t="s">
         <v>30</v>
@@ -7813,13 +7810,13 @@
         <v>35</v>
       </c>
       <c r="E36" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F36" t="s">
         <v>277</v>
       </c>
       <c r="W36" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AW36" t="s">
         <v>31</v>
@@ -7918,20 +7915,20 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 K7:K10 F7:F10 Q14:Q19 Q7 C7:C13 X7:X9 AB8:AB14 AB16:AB17" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AW46 Q14:Q19 Q7 B7:B15 X7:X9 AB15:AB16 K7:K8 AB8:AB13 F7:F12" xr:uid="{14BC2D73-1395-4E2C-9D1E-55C781825C64}">
       <formula1>$AW$30:$AW$45</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N7:N10 T14:T19 T7" xr:uid="{727A5344-B28A-4866-9EC1-7C96029AF8B6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T14:T19 T7 N7:N8" xr:uid="{727A5344-B28A-4866-9EC1-7C96029AF8B6}">
       <formula1>$AY$31:$AY$34</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7:H10" xr:uid="{FFFA1AF2-B35F-4BAA-AEF6-4A6121806F8D}">
-      <formula1>$BA$30:$BA$47</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U21:U22" xr:uid="{843CAB93-5FB8-4584-AA77-D87D9BF50E6D}">
       <formula1>"HrTim,Tim"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U7 U12:U19" xr:uid="{2E700A6E-F322-4D4F-87DE-D704594A5EA0}">
       <formula1>"HrTim,BscTim,AdvTim"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7:H12" xr:uid="{FFFA1AF2-B35F-4BAA-AEF6-4A6121806F8D}">
+      <formula1>$BA$30:$BA$47</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7957,13 +7954,13 @@
           <x14:formula1>
             <xm:f>General_Info!$P$34:$P$39</xm:f>
           </x14:formula1>
-          <xm:sqref>J7:J10 E7:E10 P14:P19 P7 B7:B13 W7:W9 AA8:AA14 AA16:AA17</xm:sqref>
+          <xm:sqref>P14:P19 P7 A7:A15 W7:W9 AA15:AA16 J7:J8 AA8:AA13 E7:E12</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C428027-B16D-4B04-9CB2-8290577ED0FB}">
           <x14:formula1>
             <xm:f>General_Info!$V$41:$V$45</xm:f>
           </x14:formula1>
-          <xm:sqref>G6:G10</xm:sqref>
+          <xm:sqref>G6:G12</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -7987,7 +7984,7 @@
         <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
@@ -7998,10 +7995,10 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G4" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
@@ -8012,7 +8009,7 @@
         <v>45</v>
       </c>
       <c r="F5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="G5" t="s">
         <v>6</v>
@@ -8026,7 +8023,7 @@
         <v>45</v>
       </c>
       <c r="F6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="G6" t="s">
         <v>7</v>
@@ -8034,7 +8031,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G7" t="s">
         <v>8</v>
@@ -8042,7 +8039,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="G8" t="s">
         <v>4</v>
@@ -8050,7 +8047,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="G9" t="s">
         <v>251</v>
@@ -8058,7 +8055,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G10" t="s">
         <v>5</v>
@@ -8066,7 +8063,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G11" t="s">
         <v>252</v>
@@ -8074,7 +8071,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="G12" t="s">
         <v>253</v>
@@ -8082,7 +8079,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="G13" t="s">
         <v>254</v>
@@ -8090,7 +8087,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="G14" t="s">
         <v>255</v>
@@ -8098,7 +8095,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F15" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G15" t="s">
         <v>256</v>
@@ -8106,7 +8103,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.3">
       <c r="F16" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="G16" t="s">
         <v>256</v>
@@ -8114,7 +8111,7 @@
     </row>
     <row r="17" spans="6:7" x14ac:dyDescent="0.3">
       <c r="F17" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G17" t="s">
         <v>256</v>
@@ -8145,37 +8142,37 @@
     </row>
     <row r="6" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y6" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y7" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="8" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y8" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="9" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y9" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="10" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y10" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="11" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y11" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="12" spans="25:25" x14ac:dyDescent="0.3">
       <c r="Y12" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -8252,7 +8249,7 @@
         <v>110</v>
       </c>
       <c r="S4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="T4" t="s">
         <v>268</v>
@@ -8278,7 +8275,7 @@
         <v>98</v>
       </c>
       <c r="S5" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="T5" t="s">
         <v>268</v>
@@ -8292,7 +8289,7 @@
     </row>
     <row r="6" spans="5:22" x14ac:dyDescent="0.3">
       <c r="S6" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="T6" t="s">
         <v>268</v>
@@ -8306,10 +8303,10 @@
     </row>
     <row r="7" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E7" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="S7" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="T7" t="s">
         <v>268</v>
@@ -8323,13 +8320,13 @@
     </row>
     <row r="8" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="S8" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="T8" t="s">
         <v>268</v>
@@ -8343,34 +8340,34 @@
     </row>
     <row r="9" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E9" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="F9" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="10" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E10" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="11" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E11" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="F11" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="12" spans="5:22" x14ac:dyDescent="0.3">
       <c r="E12" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F12" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
   </sheetData>
@@ -8417,50 +8414,50 @@
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
+        <v>332</v>
+      </c>
+      <c r="C2" t="s">
         <v>333</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>334</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>335</v>
       </c>
-      <c r="E2" t="s">
-        <v>336</v>
-      </c>
       <c r="J2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
+        <v>329</v>
+      </c>
+      <c r="C3" t="s">
         <v>330</v>
       </c>
-      <c r="C3" t="s">
-        <v>331</v>
-      </c>
       <c r="D3" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E3" t="s">
         <v>69</v>
       </c>
       <c r="J3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="K3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="P3" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D4" t="s">
         <v>50</v>
@@ -8469,13 +8466,13 @@
         <v>69</v>
       </c>
       <c r="J4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="K4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L4" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="P4" t="s">
         <v>233</v>
@@ -8483,10 +8480,10 @@
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D5" t="s">
         <v>92</v>
@@ -8495,183 +8492,207 @@
         <v>69</v>
       </c>
       <c r="J5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="K5" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>338</v>
+        <v>398</v>
       </c>
       <c r="C6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
         <v>69</v>
       </c>
       <c r="J6" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="K6" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>339</v>
+        <v>399</v>
       </c>
       <c r="C7" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>336</v>
       </c>
       <c r="E7" t="s">
         <v>69</v>
       </c>
       <c r="J7" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="K7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="C8" t="s">
         <v>331</v>
       </c>
       <c r="D8" t="s">
-        <v>341</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
         <v>69</v>
       </c>
       <c r="J8" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="K8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C9" t="s">
         <v>331</v>
       </c>
       <c r="D9" t="s">
-        <v>343</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
         <v>69</v>
       </c>
       <c r="J9" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="K9" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>404</v>
+        <v>339</v>
       </c>
       <c r="C10" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>340</v>
       </c>
       <c r="E10" t="s">
         <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="K10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>405</v>
+        <v>341</v>
       </c>
       <c r="C11" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D11" t="s">
-        <v>45</v>
+        <v>342</v>
       </c>
       <c r="E11" t="s">
         <v>69</v>
       </c>
       <c r="J11" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="K11" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>429</v>
+        <v>403</v>
       </c>
       <c r="C12" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D12" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" t="s">
+        <v>69</v>
+      </c>
+      <c r="J12" t="s">
+        <v>380</v>
+      </c>
+      <c r="K12" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>404</v>
+      </c>
+      <c r="C13" t="s">
+        <v>330</v>
+      </c>
+      <c r="D13" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" t="s">
+        <v>69</v>
+      </c>
+      <c r="J13" t="s">
+        <v>381</v>
+      </c>
+      <c r="K13" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>428</v>
+      </c>
+      <c r="C14" t="s">
+        <v>331</v>
+      </c>
+      <c r="D14" t="s">
         <v>92</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="J12" t="s">
-        <v>381</v>
-      </c>
-      <c r="K12" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="J13" t="s">
+      <c r="J14" t="s">
         <v>382</v>
-      </c>
-      <c r="K13" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="J14" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J15" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J16" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J17" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="18" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J18" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>
@@ -8691,47 +8712,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>
@@ -8761,28 +8782,28 @@
   <sheetData>
     <row r="2" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E2" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="G2" t="s">
+        <v>417</v>
+      </c>
+      <c r="H2" t="s">
         <v>418</v>
       </c>
-      <c r="H2" t="s">
-        <v>419</v>
-      </c>
       <c r="I2" t="s">
+        <v>284</v>
+      </c>
+      <c r="J2" t="s">
         <v>285</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>286</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>287</v>
-      </c>
-      <c r="L2" t="s">
-        <v>288</v>
       </c>
       <c r="M2" t="s">
         <v>42</v>
@@ -8793,7 +8814,7 @@
         <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -8814,7 +8835,7 @@
         <v>29</v>
       </c>
       <c r="M3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="4" spans="5:13" x14ac:dyDescent="0.3">
@@ -8822,7 +8843,7 @@
         <v>79</v>
       </c>
       <c r="F4" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="G4">
         <v>256</v>
@@ -8843,7 +8864,7 @@
         <v>27</v>
       </c>
       <c r="M4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="5" spans="5:13" x14ac:dyDescent="0.3">
@@ -8851,7 +8872,7 @@
         <v>219</v>
       </c>
       <c r="F5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I5" t="s">
         <v>259</v>
@@ -8866,7 +8887,7 @@
         <v>31</v>
       </c>
       <c r="M5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="6" spans="5:13" x14ac:dyDescent="0.3">
@@ -8874,7 +8895,7 @@
         <v>277</v>
       </c>
       <c r="F6" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G6">
         <v>256</v>
@@ -8895,7 +8916,7 @@
         <v>33</v>
       </c>
       <c r="M6" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="7" spans="5:13" x14ac:dyDescent="0.3">
@@ -8903,7 +8924,7 @@
         <v>278</v>
       </c>
       <c r="F7" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -8924,7 +8945,7 @@
         <v>35</v>
       </c>
       <c r="M7" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
   </sheetData>
@@ -8951,7 +8972,7 @@
   <sheetData>
     <row r="1" spans="3:14" ht="93.6" x14ac:dyDescent="1.75">
       <c r="D1" s="6" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" spans="3:14" x14ac:dyDescent="0.3">
@@ -8961,10 +8982,10 @@
     </row>
     <row r="4" spans="3:14" x14ac:dyDescent="0.3">
       <c r="L4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="N4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="5" spans="3:14" x14ac:dyDescent="0.3">
@@ -8977,19 +8998,19 @@
     </row>
     <row r="7" spans="3:14" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
+        <v>308</v>
+      </c>
+      <c r="E7" t="s">
+        <v>307</v>
+      </c>
+      <c r="F7" t="s">
+        <v>305</v>
+      </c>
+      <c r="G7" t="s">
+        <v>306</v>
+      </c>
+      <c r="J7" t="s">
         <v>309</v>
-      </c>
-      <c r="E7" t="s">
-        <v>308</v>
-      </c>
-      <c r="F7" t="s">
-        <v>306</v>
-      </c>
-      <c r="G7" t="s">
-        <v>307</v>
-      </c>
-      <c r="J7" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="8" spans="3:14" x14ac:dyDescent="0.3">
@@ -9011,7 +9032,7 @@
         <v>6000.2906390778307</v>
       </c>
       <c r="M8" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="9" spans="3:14" x14ac:dyDescent="0.3">
@@ -9022,7 +9043,7 @@
     </row>
     <row r="12" spans="3:14" x14ac:dyDescent="0.3">
       <c r="L12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" spans="3:14" x14ac:dyDescent="0.3">
@@ -9031,7 +9052,7 @@
         <v>35.998312579097856</v>
       </c>
       <c r="J13" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="L13">
         <f>L5+(L5/J15)*M9</f>
@@ -9061,10 +9082,10 @@
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.3">
       <c r="J17" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="L17" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.3">
@@ -9099,10 +9120,10 @@
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D28" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="K28" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.3">
@@ -9114,39 +9135,39 @@
         <v>0.5</v>
       </c>
       <c r="M29" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D30" t="s">
+        <v>318</v>
+      </c>
+      <c r="E30" t="s">
         <v>319</v>
       </c>
-      <c r="E30" t="s">
-        <v>320</v>
-      </c>
       <c r="F30" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="G30" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I30" t="s">
+        <v>325</v>
+      </c>
+      <c r="J30" t="s">
+        <v>323</v>
+      </c>
+      <c r="K30" t="s">
         <v>326</v>
       </c>
-      <c r="J30" t="s">
+      <c r="L30" t="s">
+        <v>327</v>
+      </c>
+      <c r="M30" t="s">
         <v>324</v>
       </c>
-      <c r="K30" t="s">
-        <v>327</v>
-      </c>
-      <c r="L30" t="s">
+      <c r="O30" t="s">
         <v>328</v>
-      </c>
-      <c r="M30" t="s">
-        <v>325</v>
-      </c>
-      <c r="O30" t="s">
-        <v>329</v>
       </c>
       <c r="P30" t="e">
         <f>2^#REF!</f>

</xml_diff>